<commit_message>
feat (test): thêm 1 nùi test case hog liệt kê hết dược
</commit_message>
<xml_diff>
--- a/English_App_Backend_TestCases.xlsx
+++ b/English_App_Backend_TestCases.xlsx
@@ -422,12 +422,12 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:F12"/>
   <cols>
-    <col min="1" max="1" width="15.83203125" customWidth="1"/>
-    <col min="2" max="2" width="45.83203125" customWidth="1"/>
-    <col min="3" max="3" width="35.83203125" customWidth="1"/>
+    <col min="1" max="1" width="18.83203125" customWidth="1"/>
+    <col min="2" max="2" width="48.83203125" customWidth="1"/>
+    <col min="3" max="3" width="40.83203125" customWidth="1"/>
     <col min="4" max="4" width="45.83203125" customWidth="1"/>
     <col min="5" max="5" width="35.83203125" customWidth="1"/>
-    <col min="6" max="6" width="45.83203125" customWidth="1"/>
+    <col min="6" max="6" width="48.83203125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -546,7 +546,7 @@
         <v>Hai bài viết gửi chấm song song</v>
       </c>
       <c r="C6" t="str">
-        <v>Kiểm thử mất kết nối mạng &amp; Lỗi hệ thống (Network &amp; System Error)</v>
+        <v>Kiểm thử đụng độ đồng thời (Concurrency / Race Condition - Update vs Delete)</v>
       </c>
       <c r="D6" t="str" xml:space="preserve">
         <v xml:space="preserve">1. Khởi tạo Service với Mock Repository / Prisma Client.
@@ -557,7 +557,7 @@
         <v>Dữ liệu test fixture trong AI.mock.ts</v>
       </c>
       <c r="F6" t="str">
-        <v>Ném ngoại lệ lỗi kết nối hoặc Rollback Transaction, không lưu dữ liệu rác.</v>
+        <v>Hệ thống phân giải đụng độ an toàn: phát hiện bản ghi đã bị xóa (P2025/404) hoặc cập nhật nguyên tử, không sinh trạng thái zombie.</v>
       </c>
     </row>
     <row r="7" xml:space="preserve">
@@ -568,7 +568,7 @@
         <v>Mất kết nối Ollama service (ECONNREFUSED) ném lỗi hệ thống</v>
       </c>
       <c r="C7" t="str">
-        <v>Kiểm thử mất kết nối mạng &amp; Lỗi hệ thống (Network &amp; System Error)</v>
+        <v>Kiểm thử đụng độ đồng thời (Concurrency / Race Condition - Update vs Delete)</v>
       </c>
       <c r="D7" t="str" xml:space="preserve">
         <v xml:space="preserve">1. Khởi tạo Service với Mock Repository / Prisma Client.
@@ -703,12 +703,12 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:F14"/>
   <cols>
-    <col min="1" max="1" width="15.83203125" customWidth="1"/>
-    <col min="2" max="2" width="45.83203125" customWidth="1"/>
-    <col min="3" max="3" width="35.83203125" customWidth="1"/>
+    <col min="1" max="1" width="18.83203125" customWidth="1"/>
+    <col min="2" max="2" width="48.83203125" customWidth="1"/>
+    <col min="3" max="3" width="40.83203125" customWidth="1"/>
     <col min="4" max="4" width="45.83203125" customWidth="1"/>
     <col min="5" max="5" width="35.83203125" customWidth="1"/>
-    <col min="6" max="6" width="45.83203125" customWidth="1"/>
+    <col min="6" max="6" width="48.83203125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -764,12 +764,12 @@
         <v>Kiểm thử chức năng chuẩn (Happy Path)</v>
       </c>
       <c r="D3" t="str" xml:space="preserve">
-        <v xml:space="preserve">1. Khởi tạo Service với Mock Repository / Prisma Client.
-2. Kích hoạt hàm nghiệp vụ tương ứng của game.
-3. Kiểm tra giá trị trả về hoặc bắt exception.</v>
+        <v xml:space="preserve">1. Thiết lập Mock Repository / Database cho Service.
+2. Gọi method service.updateSettings() với tham số kiểm thử.
+3. Đối soát kết quả hoặc mã lỗi phát sinh.</v>
       </c>
       <c r="E3" t="str">
-        <v>Dữ liệu test fixture trong game.mock.ts</v>
+        <v>Args: 1, { settings: [{ difficulty: 'EASY', itemCount: 8, pointsPerItem: 15 }] as any, }</v>
       </c>
       <c r="F3" t="str">
         <v>Hàm thực thi thành công, trả về đúng kiểu dữ liệu, các phương thức mock được gọi đúng tham số.</v>
@@ -893,7 +893,7 @@
         <v>Mất kết nối database khi truy vấn từ vựng ném lỗi</v>
       </c>
       <c r="C9" t="str">
-        <v>Kiểm thử mất kết nối mạng &amp; Lỗi hệ thống (Network &amp; System Error)</v>
+        <v>Kiểm thử đụng độ đồng thời (Concurrency / Race Condition - Update vs Delete)</v>
       </c>
       <c r="D9" t="str" xml:space="preserve">
         <v xml:space="preserve">1. Thiết lập Mock Repository / Database cho Service.
@@ -1028,12 +1028,12 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:F14"/>
   <cols>
-    <col min="1" max="1" width="15.83203125" customWidth="1"/>
-    <col min="2" max="2" width="45.83203125" customWidth="1"/>
-    <col min="3" max="3" width="35.83203125" customWidth="1"/>
+    <col min="1" max="1" width="18.83203125" customWidth="1"/>
+    <col min="2" max="2" width="48.83203125" customWidth="1"/>
+    <col min="3" max="3" width="40.83203125" customWidth="1"/>
     <col min="4" max="4" width="45.83203125" customWidth="1"/>
     <col min="5" max="5" width="35.83203125" customWidth="1"/>
-    <col min="6" max="6" width="45.83203125" customWidth="1"/>
+    <col min="6" max="6" width="48.83203125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1174,7 +1174,7 @@
         <v>Thêm nhiều nhóm liên tiếp bảo toàn mảng dữ liệu trong bộ nhớ</v>
       </c>
       <c r="C7" t="str">
-        <v>Kiểm thử đụng độ đồng thời (Concurrency / Race Condition)</v>
+        <v>Kiểm thử đụng độ đồng thời (Concurrency / Race Condition - Update vs Delete)</v>
       </c>
       <c r="D7" t="str" xml:space="preserve">
         <v xml:space="preserve">1. Thiết lập Mock Repository / Database cho Service.
@@ -1185,7 +1185,7 @@
         <v>Args: 'Nhóm Song Song 1', ['a']</v>
       </c>
       <c r="F7" t="str">
-        <v>Hàm thực thi thành công, trả về đúng kiểu dữ liệu, các phương thức mock được gọi đúng tham số.</v>
+        <v>Hệ thống phân giải đụng độ an toàn: phát hiện bản ghi đã bị xóa (P2025/404) hoặc cập nhật nguyên tử, không sinh trạng thái zombie.</v>
       </c>
     </row>
     <row r="8" xml:space="preserve">
@@ -1196,7 +1196,7 @@
         <v>Chặn tạo nhóm trùng tên với nhóm đã tồn tại (case-insensitive)</v>
       </c>
       <c r="C8" t="str">
-        <v>Kiểm thử toàn vẹn dữ liệu &amp; Xung đột (Data Conflict / Rollback)</v>
+        <v>Kiểm thử phân quyền &amp; Bảo mật (Authorization &amp; Security 401/403)</v>
       </c>
       <c r="D8" t="str" xml:space="preserve">
         <v xml:space="preserve">1. Thiết lập Mock Repository / Database cho Service.
@@ -1270,10 +1270,10 @@
 3. Xác thực mã trạng thái HTTP và cấu trúc JSON trả về.</v>
       </c>
       <c r="E11" t="str">
-        <v>Path param hoặc Payload chuẩn của keyword-setting</v>
+        <v>{ group: 'Khoa học', keywords: ['science', 'research'] }</v>
       </c>
       <c r="F11" t="str">
-        <v>HTTP Status: 200. Response trả về success = true cùng dữ liệu hợp lệ.</v>
+        <v>HTTP Status: 201. Response trả về success = true cùng dữ liệu hợp lệ.</v>
       </c>
     </row>
     <row r="12" xml:space="preserve">
@@ -1314,10 +1314,10 @@
 3. Xác thực mã trạng thái HTTP và cấu trúc JSON trả về.</v>
       </c>
       <c r="E13" t="str">
-        <v>Path param hoặc Payload chuẩn của keyword-setting</v>
+        <v>{ group: 'Trùng', keywords: ['a'] }</v>
       </c>
       <c r="F13" t="str">
-        <v>HTTP Status: 200. Response trả về success = true cùng dữ liệu hợp lệ.</v>
+        <v>HTTP Status: 400. Báo lỗi validation hoặc bad request rõ ràng, không làm crash server.</v>
       </c>
     </row>
     <row r="14" xml:space="preserve">
@@ -1328,7 +1328,7 @@
         <v>2 request thêm nhóm song song</v>
       </c>
       <c r="C14" t="str">
-        <v>Kiểm thử đụng độ đồng thời (Concurrency / Race Condition)</v>
+        <v>Kiểm thử đụng độ đồng thời (Concurrency / Race Condition - Update vs Delete)</v>
       </c>
       <c r="D14" t="str" xml:space="preserve">
         <v xml:space="preserve">1. Thiết lập phiên đăng nhập / Mock quyền truy cập tương ứng.
@@ -1353,12 +1353,12 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:F7"/>
   <cols>
-    <col min="1" max="1" width="15.83203125" customWidth="1"/>
-    <col min="2" max="2" width="45.83203125" customWidth="1"/>
-    <col min="3" max="3" width="35.83203125" customWidth="1"/>
+    <col min="1" max="1" width="18.83203125" customWidth="1"/>
+    <col min="2" max="2" width="48.83203125" customWidth="1"/>
+    <col min="3" max="3" width="40.83203125" customWidth="1"/>
     <col min="4" max="4" width="45.83203125" customWidth="1"/>
     <col min="5" max="5" width="35.83203125" customWidth="1"/>
-    <col min="6" max="6" width="45.83203125" customWidth="1"/>
+    <col min="6" max="6" width="48.83203125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1433,7 +1433,7 @@
         <v>Nhiều học viên cùng tải bảng xếp hạng song song</v>
       </c>
       <c r="C4" t="str">
-        <v>Kiểm thử đụng độ đồng thời (Concurrency / Race Condition)</v>
+        <v>Kiểm thử đụng độ đồng thời (Concurrency / Race Condition - Update vs Delete)</v>
       </c>
       <c r="D4" t="str" xml:space="preserve">
         <v xml:space="preserve">1. Thiết lập Mock Repository / Database cho Service.
@@ -1444,7 +1444,7 @@
         <v>Args: 1, 10</v>
       </c>
       <c r="F4" t="str">
-        <v>Hàm thực thi thành công, trả về đúng kiểu dữ liệu, các phương thức mock được gọi đúng tham số.</v>
+        <v>Hệ thống phân giải đụng độ an toàn: phát hiện bản ghi đã bị xóa (P2025/404) hoặc cập nhật nguyên tử, không sinh trạng thái zombie.</v>
       </c>
     </row>
     <row r="5" xml:space="preserve">
@@ -1455,7 +1455,7 @@
         <v>Mất kết nối DB khi lấy BXH ném lỗi hệ thống</v>
       </c>
       <c r="C5" t="str">
-        <v>Kiểm thử mất kết nối mạng &amp; Lỗi hệ thống (Network &amp; System Error)</v>
+        <v>Kiểm thử toàn vẹn dữ liệu &amp; Xung đột (Data Conflict / Rollback)</v>
       </c>
       <c r="D5" t="str" xml:space="preserve">
         <v xml:space="preserve">1. Thiết lập Mock Repository / Database cho Service.
@@ -1524,12 +1524,12 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:F14"/>
   <cols>
-    <col min="1" max="1" width="15.83203125" customWidth="1"/>
-    <col min="2" max="2" width="45.83203125" customWidth="1"/>
-    <col min="3" max="3" width="35.83203125" customWidth="1"/>
+    <col min="1" max="1" width="18.83203125" customWidth="1"/>
+    <col min="2" max="2" width="48.83203125" customWidth="1"/>
+    <col min="3" max="3" width="40.83203125" customWidth="1"/>
     <col min="4" max="4" width="45.83203125" customWidth="1"/>
     <col min="5" max="5" width="35.83203125" customWidth="1"/>
-    <col min="6" max="6" width="45.83203125" customWidth="1"/>
+    <col min="6" max="6" width="48.83203125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1607,12 +1607,12 @@
         <v>Kiểm thử chức năng chuẩn (Happy Path)</v>
       </c>
       <c r="D4" t="str" xml:space="preserve">
-        <v xml:space="preserve">1. Khởi tạo Service với Mock Repository / Prisma Client.
-2. Kích hoạt hàm nghiệp vụ tương ứng của mario-game.
-3. Kiểm tra giá trị trả về hoặc bắt exception.</v>
+        <v xml:space="preserve">1. Thiết lập Mock Repository / Database cho Service.
+2. Gọi method service.finishGame() với tham số kiểm thử.
+3. Đối soát kết quả hoặc mã lỗi phát sinh.</v>
       </c>
       <c r="E4" t="str">
-        <v>Dữ liệu test fixture trong mario-game.mock.ts</v>
+        <v>Args: 1, mockMarioFinishGameInput</v>
       </c>
       <c r="F4" t="str">
         <v>Hàm thực thi thành công, trả về đúng kiểu dữ liệu, các phương thức mock được gọi đúng tham số.</v>
@@ -1670,7 +1670,7 @@
         <v>Hai request chốt điểm finishGame gửi đồng thời</v>
       </c>
       <c r="C7" t="str">
-        <v>Kiểm thử mất kết nối mạng &amp; Lỗi hệ thống (Network &amp; System Error)</v>
+        <v>Kiểm thử đụng độ đồng thời (Concurrency / Race Condition - Update vs Delete)</v>
       </c>
       <c r="D7" t="str" xml:space="preserve">
         <v xml:space="preserve">1. Thiết lập Mock Repository / Database cho Service.
@@ -1681,7 +1681,7 @@
         <v>Args: 1, mockMarioFinishGameInput</v>
       </c>
       <c r="F7" t="str">
-        <v>Ném ngoại lệ lỗi kết nối hoặc Rollback Transaction, không lưu dữ liệu rác.</v>
+        <v>Hệ thống phân giải đụng độ an toàn: phát hiện bản ghi đã bị xóa (P2025/404) hoặc cập nhật nguyên tử, không sinh trạng thái zombie.</v>
       </c>
     </row>
     <row r="8" xml:space="preserve">
@@ -1692,7 +1692,7 @@
         <v>Mất kết nối DB khi lưu tiến trình ném lỗi</v>
       </c>
       <c r="C8" t="str">
-        <v>Kiểm thử mất kết nối mạng &amp; Lỗi hệ thống (Network &amp; System Error)</v>
+        <v>Kiểm thử đụng độ đồng thời (Concurrency / Race Condition - Update vs Delete)</v>
       </c>
       <c r="D8" t="str" xml:space="preserve">
         <v xml:space="preserve">1. Thiết lập Mock Repository / Database cho Service.
@@ -1718,11 +1718,11 @@
       </c>
       <c r="D9" t="str" xml:space="preserve">
         <v xml:space="preserve">1. Thiết lập phiên đăng nhập / Mock quyền truy cập tương ứng.
-2. Gửi request HTTP GET tới endpoint /api/mario-game/start.
+2. Gửi request HTTP GET tới endpoint /api/mario-game/start?limit=4.
 3. Xác thực mã trạng thái HTTP và cấu trúc JSON trả về.</v>
       </c>
       <c r="E9" t="str">
-        <v>Path param hoặc Payload chuẩn của mario-game</v>
+        <v>Query parameters: limit=4</v>
       </c>
       <c r="F9" t="str">
         <v>HTTP Status: 200. Response trả về success = true cùng dữ liệu hợp lệ.</v>
@@ -1744,7 +1744,7 @@
 3. Xác thực mã trạng thái HTTP và cấu trúc JSON trả về.</v>
       </c>
       <c r="E10" t="str">
-        <v>Path param hoặc Payload chuẩn của mario-game</v>
+        <v>mockMarioMatchPairInput</v>
       </c>
       <c r="F10" t="str">
         <v>HTTP Status: 200. Response trả về success = true cùng dữ liệu hợp lệ.</v>
@@ -1824,7 +1824,7 @@
         <v>Lỗi database khi kết thúc ván trả về 500</v>
       </c>
       <c r="C14" t="str">
-        <v>Kiểm thử mất kết nối mạng &amp; Lỗi hệ thống (Network &amp; System Error)</v>
+        <v>Kiểm thử trường hợp biên &amp; Ngoại lệ (Negative / Bad Case)</v>
       </c>
       <c r="D14" t="str" xml:space="preserve">
         <v xml:space="preserve">1. Thiết lập phiên đăng nhập / Mock quyền truy cập tương ứng.
@@ -1849,12 +1849,12 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:F14"/>
   <cols>
-    <col min="1" max="1" width="15.83203125" customWidth="1"/>
-    <col min="2" max="2" width="45.83203125" customWidth="1"/>
-    <col min="3" max="3" width="35.83203125" customWidth="1"/>
+    <col min="1" max="1" width="18.83203125" customWidth="1"/>
+    <col min="2" max="2" width="48.83203125" customWidth="1"/>
+    <col min="3" max="3" width="40.83203125" customWidth="1"/>
     <col min="4" max="4" width="45.83203125" customWidth="1"/>
     <col min="5" max="5" width="35.83203125" customWidth="1"/>
-    <col min="6" max="6" width="45.83203125" customWidth="1"/>
+    <col min="6" max="6" width="48.83203125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1932,12 +1932,12 @@
         <v>Kiểm thử chức năng chuẩn (Happy Path)</v>
       </c>
       <c r="D4" t="str" xml:space="preserve">
-        <v xml:space="preserve">1. Khởi tạo Service với Mock Repository / Prisma Client.
-2. Kích hoạt hàm nghiệp vụ tương ứng của memory-card.
-3. Kiểm tra giá trị trả về hoặc bắt exception.</v>
+        <v xml:space="preserve">1. Thiết lập Mock Repository / Database cho Service.
+2. Gọi method service.finishGame() với tham số kiểm thử.
+3. Đối soát kết quả hoặc mã lỗi phát sinh.</v>
       </c>
       <c r="E4" t="str">
-        <v>Dữ liệu test fixture trong memory-card.mock.ts</v>
+        <v>Args: 1, mockFinishMemoryInput</v>
       </c>
       <c r="F4" t="str">
         <v>Hàm thực thi thành công, trả về đúng kiểu dữ liệu, các phương thức mock được gọi đúng tham số.</v>
@@ -1995,7 +1995,7 @@
         <v>Hai request chốt điểm Memory Card song song</v>
       </c>
       <c r="C7" t="str">
-        <v>Kiểm thử mất kết nối mạng &amp; Lỗi hệ thống (Network &amp; System Error)</v>
+        <v>Kiểm thử đụng độ đồng thời (Concurrency / Race Condition - Update vs Delete)</v>
       </c>
       <c r="D7" t="str" xml:space="preserve">
         <v xml:space="preserve">1. Thiết lập Mock Repository / Database cho Service.
@@ -2006,7 +2006,7 @@
         <v>Args: 1, mockFinishMemoryInput</v>
       </c>
       <c r="F7" t="str">
-        <v>Ném ngoại lệ lỗi kết nối hoặc Rollback Transaction, không lưu dữ liệu rác.</v>
+        <v>Hệ thống phân giải đụng độ an toàn: phát hiện bản ghi đã bị xóa (P2025/404) hoặc cập nhật nguyên tử, không sinh trạng thái zombie.</v>
       </c>
     </row>
     <row r="8" xml:space="preserve">
@@ -2017,7 +2017,7 @@
         <v>Mất kết nối database khi lưu tiến trình ném lỗi</v>
       </c>
       <c r="C8" t="str">
-        <v>Kiểm thử mất kết nối mạng &amp; Lỗi hệ thống (Network &amp; System Error)</v>
+        <v>Kiểm thử đụng độ đồng thời (Concurrency / Race Condition - Update vs Delete)</v>
       </c>
       <c r="D8" t="str" xml:space="preserve">
         <v xml:space="preserve">1. Thiết lập Mock Repository / Database cho Service.
@@ -2069,7 +2069,7 @@
 3. Xác thực mã trạng thái HTTP và cấu trúc JSON trả về.</v>
       </c>
       <c r="E10" t="str">
-        <v>Path param hoặc Payload chuẩn của memory-card</v>
+        <v>mockSaveMemoryProgressInput</v>
       </c>
       <c r="F10" t="str">
         <v>HTTP Status: 200. Response trả về success = true cùng dữ liệu hợp lệ.</v>
@@ -2091,7 +2091,7 @@
 3. Xác thực mã trạng thái HTTP và cấu trúc JSON trả về.</v>
       </c>
       <c r="E11" t="str">
-        <v>Path param hoặc Payload chuẩn của memory-card</v>
+        <v>mockFinishMemoryInput</v>
       </c>
       <c r="F11" t="str">
         <v>HTTP Status: 200. Response trả về success = true cùng dữ liệu hợp lệ.</v>
@@ -2149,7 +2149,7 @@
         <v>Lỗi database khi kết thúc ván trả về 500</v>
       </c>
       <c r="C14" t="str">
-        <v>Kiểm thử mất kết nối mạng &amp; Lỗi hệ thống (Network &amp; System Error)</v>
+        <v>Kiểm thử trường hợp biên &amp; Ngoại lệ (Negative / Bad Case)</v>
       </c>
       <c r="D14" t="str" xml:space="preserve">
         <v xml:space="preserve">1. Thiết lập phiên đăng nhập / Mock quyền truy cập tương ứng.
@@ -2174,12 +2174,12 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:F12"/>
   <cols>
-    <col min="1" max="1" width="15.83203125" customWidth="1"/>
-    <col min="2" max="2" width="45.83203125" customWidth="1"/>
-    <col min="3" max="3" width="35.83203125" customWidth="1"/>
+    <col min="1" max="1" width="18.83203125" customWidth="1"/>
+    <col min="2" max="2" width="48.83203125" customWidth="1"/>
+    <col min="3" max="3" width="40.83203125" customWidth="1"/>
     <col min="4" max="4" width="45.83203125" customWidth="1"/>
     <col min="5" max="5" width="35.83203125" customWidth="1"/>
-    <col min="6" max="6" width="45.83203125" customWidth="1"/>
+    <col min="6" max="6" width="48.83203125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -2298,7 +2298,7 @@
         <v>Đánh dấu thông báo không thuộc quyền sở hữu (IDOR check: userId khác) không làm ảnh hưởng bản ghi</v>
       </c>
       <c r="C6" t="str">
-        <v>Kiểm thử trường hợp biên &amp; Ngoại lệ (Negative / Bad Case)</v>
+        <v>Kiểm thử phân quyền &amp; Bảo mật (Authorization &amp; Security 401/403)</v>
       </c>
       <c r="D6" t="str" xml:space="preserve">
         <v xml:space="preserve">1. Thiết lập Mock Repository / Database cho Service.
@@ -2309,7 +2309,7 @@
         <v>Args: 999, 1</v>
       </c>
       <c r="F6" t="str">
-        <v>Ném ngoại lệ ApiError với status 4xx, mã lỗi 'ApiError'.</v>
+        <v>Hàm thực thi thành công, trả về đúng kiểu dữ liệu, các phương thức mock được gọi đúng tham số.</v>
       </c>
     </row>
     <row r="7" xml:space="preserve">
@@ -2320,7 +2320,7 @@
         <v>Nhiều tiến trình cùng gửi thông báo cho Admin đồng thời</v>
       </c>
       <c r="C7" t="str">
-        <v>Kiểm thử đụng độ đồng thời (Concurrency / Race Condition)</v>
+        <v>Kiểm thử đụng độ đồng thời (Concurrency / Race Condition - Update vs Delete)</v>
       </c>
       <c r="D7" t="str" xml:space="preserve">
         <v xml:space="preserve">1. Thiết lập Mock Repository / Database cho Service.
@@ -2331,7 +2331,7 @@
         <v>Args: 'T1', 'B1'</v>
       </c>
       <c r="F7" t="str">
-        <v>Hàm thực thi thành công, trả về đúng kiểu dữ liệu, các phương thức mock được gọi đúng tham số.</v>
+        <v>Hệ thống phân giải đụng độ an toàn: phát hiện bản ghi đã bị xóa (P2025/404) hoặc cập nhật nguyên tử, không sinh trạng thái zombie.</v>
       </c>
     </row>
     <row r="8" xml:space="preserve">
@@ -2342,7 +2342,7 @@
         <v>Mất kết nối DB khi lấy danh sách thông báo ném lỗi hệ thống</v>
       </c>
       <c r="C8" t="str">
-        <v>Kiểm thử mất kết nối mạng &amp; Lỗi hệ thống (Network &amp; System Error)</v>
+        <v>Kiểm thử toàn vẹn dữ liệu &amp; Xung đột (Data Conflict / Rollback)</v>
       </c>
       <c r="D8" t="str" xml:space="preserve">
         <v xml:space="preserve">1. Thiết lập Mock Repository / Database cho Service.
@@ -2455,12 +2455,12 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:F15"/>
   <cols>
-    <col min="1" max="1" width="15.83203125" customWidth="1"/>
-    <col min="2" max="2" width="45.83203125" customWidth="1"/>
-    <col min="3" max="3" width="35.83203125" customWidth="1"/>
+    <col min="1" max="1" width="18.83203125" customWidth="1"/>
+    <col min="2" max="2" width="48.83203125" customWidth="1"/>
+    <col min="3" max="3" width="40.83203125" customWidth="1"/>
     <col min="4" max="4" width="45.83203125" customWidth="1"/>
     <col min="5" max="5" width="35.83203125" customWidth="1"/>
-    <col min="6" max="6" width="45.83203125" customWidth="1"/>
+    <col min="6" max="6" width="48.83203125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -2579,7 +2579,7 @@
         <v>Nhiều học viên Onboarding song song không làm sai lệch ngân hàng câu hỏi</v>
       </c>
       <c r="C6" t="str">
-        <v>Kiểm thử đụng độ đồng thời (Concurrency / Race Condition)</v>
+        <v>Kiểm thử đụng độ đồng thời (Concurrency / Race Condition - Update vs Delete)</v>
       </c>
       <c r="D6" t="str" xml:space="preserve">
         <v xml:space="preserve">1. Khởi tạo Service với Mock Repository / Prisma Client.
@@ -2590,7 +2590,7 @@
         <v>Dữ liệu test fixture trong onboarding.mock.ts</v>
       </c>
       <c r="F6" t="str">
-        <v>Hàm thực thi thành công, trả về đúng kiểu dữ liệu, các phương thức mock được gọi đúng tham số.</v>
+        <v>Hệ thống phân giải đụng độ an toàn: phát hiện bản ghi đã bị xóa (P2025/404) hoặc cập nhật nguyên tử, không sinh trạng thái zombie.</v>
       </c>
     </row>
     <row r="7" xml:space="preserve">
@@ -2623,7 +2623,7 @@
         <v>Mất kết nối DB khi cập nhật kết quả user ném lỗi hệ thống</v>
       </c>
       <c r="C8" t="str">
-        <v>Kiểm thử mất kết nối mạng &amp; Lỗi hệ thống (Network &amp; System Error)</v>
+        <v>Kiểm thử trường hợp biên &amp; Ngoại lệ (Negative / Bad Case)</v>
       </c>
       <c r="D8" t="str" xml:space="preserve">
         <v xml:space="preserve">1. Khởi tạo Service với Mock Repository / Prisma Client.
@@ -2722,7 +2722,7 @@
         <v>{ job: 'Designer', interests: 'Art', // thiếu answers }</v>
       </c>
       <c r="F12" t="str">
-        <v xml:space="preserve">HTTP Status: 400 / 422. </v>
+        <v>HTTP Status: 400. Báo lỗi validation hoặc bad request rõ ràng, không làm crash server.</v>
       </c>
     </row>
     <row r="13" xml:space="preserve">
@@ -2744,7 +2744,7 @@
         <v>{ answers: 'not_an_array', }</v>
       </c>
       <c r="F13" t="str">
-        <v xml:space="preserve">HTTP Status: 400 / 422. </v>
+        <v>HTTP Status: 400. Báo lỗi validation hoặc bad request rõ ràng, không làm crash server.</v>
       </c>
     </row>
     <row r="14" xml:space="preserve">
@@ -2755,7 +2755,7 @@
         <v>Gửi 2 request submit đồng thời đều nhận được phản hồi</v>
       </c>
       <c r="C14" t="str">
-        <v>Kiểm thử đụng độ đồng thời (Concurrency / Race Condition)</v>
+        <v>Kiểm thử đụng độ đồng thời (Concurrency / Race Condition - Update vs Delete)</v>
       </c>
       <c r="D14" t="str" xml:space="preserve">
         <v xml:space="preserve">1. Thiết lập phiên đăng nhập / Mock quyền truy cập tương ứng.
@@ -2777,7 +2777,7 @@
         <v>Mất kết nối DB khi processOnboarding trả về 500 lỗi máy chủ</v>
       </c>
       <c r="C15" t="str">
-        <v>Kiểm thử mất kết nối mạng &amp; Lỗi hệ thống (Network &amp; System Error)</v>
+        <v>Kiểm thử toàn vẹn dữ liệu &amp; Xung đột (Data Conflict / Rollback)</v>
       </c>
       <c r="D15" t="str" xml:space="preserve">
         <v xml:space="preserve">1. Thiết lập phiên đăng nhập / Mock quyền truy cập tương ứng.
@@ -2802,12 +2802,12 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:F12"/>
   <cols>
-    <col min="1" max="1" width="15.83203125" customWidth="1"/>
-    <col min="2" max="2" width="45.83203125" customWidth="1"/>
-    <col min="3" max="3" width="35.83203125" customWidth="1"/>
+    <col min="1" max="1" width="18.83203125" customWidth="1"/>
+    <col min="2" max="2" width="48.83203125" customWidth="1"/>
+    <col min="3" max="3" width="40.83203125" customWidth="1"/>
     <col min="4" max="4" width="45.83203125" customWidth="1"/>
     <col min="5" max="5" width="35.83203125" customWidth="1"/>
-    <col min="6" max="6" width="45.83203125" customWidth="1"/>
+    <col min="6" max="6" width="48.83203125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -2882,7 +2882,7 @@
         <v>Chặn nhận thưởng lần 2 nếu activityLog đã ghi nhận claim hôm nay</v>
       </c>
       <c r="C4" t="str">
-        <v>Kiểm thử đụng độ đồng thời (Concurrency / Race Condition)</v>
+        <v>Kiểm thử phân quyền &amp; Bảo mật (Authorization &amp; Security 401/403)</v>
       </c>
       <c r="D4" t="str" xml:space="preserve">
         <v xml:space="preserve">1. Khởi tạo Service với Mock Repository / Prisma Client.
@@ -2926,7 +2926,7 @@
         <v>Xử lý lỗi ngắt kết nối DB khi đếm tiến độ nhiệm vụ</v>
       </c>
       <c r="C6" t="str">
-        <v>Kiểm thử mất kết nối mạng &amp; Lỗi hệ thống (Network &amp; System Error)</v>
+        <v>Kiểm thử trường hợp biên &amp; Ngoại lệ (Negative / Bad Case)</v>
       </c>
       <c r="D6" t="str" xml:space="preserve">
         <v xml:space="preserve">1. Khởi tạo Service với Mock Repository / Prisma Client.
@@ -3036,7 +3036,7 @@
         <v>POST /api/student/quests/claim đã nhận hôm nay trả về 400</v>
       </c>
       <c r="C11" t="str">
-        <v>Kiểm thử đụng độ đồng thời (Concurrency / Race Condition)</v>
+        <v>Kiểm thử đụng độ đồng thời (Concurrency / Race Condition - Update vs Delete)</v>
       </c>
       <c r="D11" t="str" xml:space="preserve">
         <v xml:space="preserve">1. Thiết lập phiên đăng nhập / Mock quyền truy cập tương ứng.
@@ -3044,10 +3044,10 @@
 3. Xác thực mã trạng thái HTTP và cấu trúc JSON trả về.</v>
       </c>
       <c r="E11" t="str">
-        <v>Path param hoặc Payload chuẩn của quest</v>
+        <v>{ questId: 'quest_login' }</v>
       </c>
       <c r="F11" t="str">
-        <v>HTTP Status: 200. Response trả về success = true cùng dữ liệu hợp lệ.</v>
+        <v>HTTP Status: 400. Báo lỗi validation hoặc bad request rõ ràng, không làm crash server.</v>
       </c>
     </row>
     <row r="12" xml:space="preserve">
@@ -3058,7 +3058,7 @@
         <v>Lỗi kết nối DB trong transaction trả về 500 lỗi máy chủ</v>
       </c>
       <c r="C12" t="str">
-        <v>Kiểm thử mất kết nối mạng &amp; Lỗi hệ thống (Network &amp; System Error)</v>
+        <v>Kiểm thử toàn vẹn dữ liệu &amp; Xung đột (Data Conflict / Rollback)</v>
       </c>
       <c r="D12" t="str" xml:space="preserve">
         <v xml:space="preserve">1. Thiết lập phiên đăng nhập / Mock quyền truy cập tương ứng.
@@ -3083,12 +3083,12 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:F13"/>
   <cols>
-    <col min="1" max="1" width="15.83203125" customWidth="1"/>
-    <col min="2" max="2" width="45.83203125" customWidth="1"/>
-    <col min="3" max="3" width="35.83203125" customWidth="1"/>
+    <col min="1" max="1" width="18.83203125" customWidth="1"/>
+    <col min="2" max="2" width="48.83203125" customWidth="1"/>
+    <col min="3" max="3" width="40.83203125" customWidth="1"/>
     <col min="4" max="4" width="45.83203125" customWidth="1"/>
     <col min="5" max="5" width="35.83203125" customWidth="1"/>
-    <col min="6" max="6" width="45.83203125" customWidth="1"/>
+    <col min="6" max="6" width="48.83203125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -3207,7 +3207,7 @@
         <v>Chống bug farm XP: Hoàn thành lại bài học đã học trước đó nhận +0 XP</v>
       </c>
       <c r="C6" t="str">
-        <v>Kiểm thử đụng độ đồng thời (Concurrency / Race Condition)</v>
+        <v>Kiểm thử đụng độ đồng thời (Concurrency / Race Condition - Update vs Delete)</v>
       </c>
       <c r="D6" t="str" xml:space="preserve">
         <v xml:space="preserve">1. Thiết lập Mock Repository / Database cho Service.
@@ -3218,7 +3218,7 @@
         <v>Args: 1, 101</v>
       </c>
       <c r="F6" t="str">
-        <v>Hàm thực thi thành công, trả về đúng kiểu dữ liệu, các phương thức mock được gọi đúng tham số.</v>
+        <v>Hệ thống phân giải đụng độ an toàn: phát hiện bản ghi đã bị xóa (P2025/404) hoặc cập nhật nguyên tử, không sinh trạng thái zombie.</v>
       </c>
     </row>
     <row r="7" xml:space="preserve">
@@ -3229,7 +3229,7 @@
         <v>Mất kết nối DB khi cộng XP ném lỗi máy chủ</v>
       </c>
       <c r="C7" t="str">
-        <v>Kiểm thử mất kết nối mạng &amp; Lỗi hệ thống (Network &amp; System Error)</v>
+        <v>Kiểm thử toàn vẹn dữ liệu &amp; Xung đột (Data Conflict / Rollback)</v>
       </c>
       <c r="D7" t="str" xml:space="preserve">
         <v xml:space="preserve">1. Thiết lập Mock Repository / Database cho Service.
@@ -3277,7 +3277,7 @@
       </c>
       <c r="D9" t="str" xml:space="preserve">
         <v xml:space="preserve">1. Thiết lập phiên đăng nhập / Mock quyền truy cập tương ứng.
-2. Gửi request HTTP POST tới endpoint /api/student/lessons/:id/complete.
+2. Gửi request HTTP POST tới endpoint /api/student/lessons/101/complete.
 3. Xác thực mã trạng thái HTTP và cấu trúc JSON trả về.</v>
       </c>
       <c r="E9" t="str">
@@ -3328,7 +3328,7 @@
         <v>Path param hoặc Payload chuẩn của student-lesson</v>
       </c>
       <c r="F11" t="str">
-        <v xml:space="preserve">HTTP Status: 404. </v>
+        <v>HTTP Status: 404. Báo lỗi student_not_found do bản ghi đã bị xóa hoặc không tồn tại.</v>
       </c>
     </row>
     <row r="12" xml:space="preserve">
@@ -3339,7 +3339,7 @@
         <v>2 request hoàn thành bài học đồng thời</v>
       </c>
       <c r="C12" t="str">
-        <v>Kiểm thử đụng độ đồng thời (Concurrency / Race Condition)</v>
+        <v>Kiểm thử đụng độ đồng thời (Concurrency / Race Condition - Update vs Delete)</v>
       </c>
       <c r="D12" t="str" xml:space="preserve">
         <v xml:space="preserve">1. Thiết lập phiên đăng nhập / Mock quyền truy cập tương ứng.
@@ -3361,7 +3361,7 @@
         <v>Lỗi kết nối DB trả về 500 lỗi máy chủ</v>
       </c>
       <c r="C13" t="str">
-        <v>Kiểm thử mất kết nối mạng &amp; Lỗi hệ thống (Network &amp; System Error)</v>
+        <v>Kiểm thử toàn vẹn dữ liệu &amp; Xung đột (Data Conflict / Rollback)</v>
       </c>
       <c r="D13" t="str" xml:space="preserve">
         <v xml:space="preserve">1. Thiết lập phiên đăng nhập / Mock quyền truy cập tương ứng.
@@ -3386,12 +3386,12 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:F13"/>
   <cols>
-    <col min="1" max="1" width="15.83203125" customWidth="1"/>
-    <col min="2" max="2" width="45.83203125" customWidth="1"/>
-    <col min="3" max="3" width="35.83203125" customWidth="1"/>
+    <col min="1" max="1" width="18.83203125" customWidth="1"/>
+    <col min="2" max="2" width="48.83203125" customWidth="1"/>
+    <col min="3" max="3" width="40.83203125" customWidth="1"/>
     <col min="4" max="4" width="45.83203125" customWidth="1"/>
     <col min="5" max="5" width="35.83203125" customWidth="1"/>
-    <col min="6" max="6" width="45.83203125" customWidth="1"/>
+    <col min="6" max="6" width="48.83203125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -3554,7 +3554,7 @@
         <v>Hai yêu cầu nộp bài đồng thời cùng lúc</v>
       </c>
       <c r="C8" t="str">
-        <v>Kiểm thử mất kết nối mạng &amp; Lỗi hệ thống (Network &amp; System Error)</v>
+        <v>Kiểm thử đụng độ đồng thời (Concurrency / Race Condition - Update vs Delete)</v>
       </c>
       <c r="D8" t="str" xml:space="preserve">
         <v xml:space="preserve">1. Thiết lập Mock Repository / Database cho Service.
@@ -3565,7 +3565,7 @@
         <v>Args: 1, 1, mockTestSubmission</v>
       </c>
       <c r="F8" t="str">
-        <v>Ném ngoại lệ lỗi kết nối hoặc Rollback Transaction, không lưu dữ liệu rác.</v>
+        <v>Hệ thống phân giải đụng độ an toàn: phát hiện bản ghi đã bị xóa (P2025/404) hoặc cập nhật nguyên tử, không sinh trạng thái zombie.</v>
       </c>
     </row>
     <row r="9" xml:space="preserve">
@@ -3576,7 +3576,7 @@
         <v>Mất kết nối database khi nộp bài thi ném lỗi</v>
       </c>
       <c r="C9" t="str">
-        <v>Kiểm thử mất kết nối mạng &amp; Lỗi hệ thống (Network &amp; System Error)</v>
+        <v>Kiểm thử đụng độ đồng thời (Concurrency / Race Condition - Update vs Delete)</v>
       </c>
       <c r="D9" t="str" xml:space="preserve">
         <v xml:space="preserve">1. Thiết lập Mock Repository / Database cho Service.
@@ -3628,7 +3628,7 @@
 3. Xác thực mã trạng thái HTTP và cấu trúc JSON trả về.</v>
       </c>
       <c r="E11" t="str">
-        <v>Path param hoặc Payload chuẩn của student-test</v>
+        <v>{ submissions: mockTestSubmission }</v>
       </c>
       <c r="F11" t="str">
         <v>HTTP Status: 200. Response trả về success = true cùng dữ liệu hợp lệ.</v>
@@ -3664,7 +3664,7 @@
         <v>Lỗi database khi nộp bài thi trả về 500</v>
       </c>
       <c r="C13" t="str">
-        <v>Kiểm thử mất kết nối mạng &amp; Lỗi hệ thống (Network &amp; System Error)</v>
+        <v>Kiểm thử trường hợp biên &amp; Ngoại lệ (Negative / Bad Case)</v>
       </c>
       <c r="D13" t="str" xml:space="preserve">
         <v xml:space="preserve">1. Thiết lập phiên đăng nhập / Mock quyền truy cập tương ứng.
@@ -3687,14 +3687,14 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F11"/>
+  <dimension ref="A1:F32"/>
   <cols>
-    <col min="1" max="1" width="15.83203125" customWidth="1"/>
-    <col min="2" max="2" width="45.83203125" customWidth="1"/>
-    <col min="3" max="3" width="35.83203125" customWidth="1"/>
+    <col min="1" max="1" width="18.83203125" customWidth="1"/>
+    <col min="2" max="2" width="48.83203125" customWidth="1"/>
+    <col min="3" max="3" width="40.83203125" customWidth="1"/>
     <col min="4" max="4" width="45.83203125" customWidth="1"/>
     <col min="5" max="5" width="35.83203125" customWidth="1"/>
-    <col min="6" max="6" width="45.83203125" customWidth="1"/>
+    <col min="6" max="6" width="48.83203125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -3728,12 +3728,12 @@
         <v>Kiểm thử chức năng chuẩn (Happy Path)</v>
       </c>
       <c r="D2" t="str" xml:space="preserve">
-        <v xml:space="preserve">1. Khởi tạo Service với Mock Repository / Prisma Client.
-2. Kích hoạt hàm nghiệp vụ tương ứng của StudentManage.
-3. Kiểm tra giá trị trả về hoặc bắt exception.</v>
+        <v xml:space="preserve">1. Thiết lập Mock Repository / Database cho Service.
+2. Gọi method service.getStudentslist() với tham số kiểm thử.
+3. Đối soát kết quả hoặc mã lỗi phát sinh.</v>
       </c>
       <c r="E2" t="str">
-        <v>Dữ liệu test fixture trong StudentManage.mock.ts</v>
+        <v>Args: { page: 1, limit: 10, sortBy: 'createdAt', sortOrder: 'desc', }</v>
       </c>
       <c r="F2" t="str">
         <v>Hàm thực thi thành công, trả về đúng kiểu dữ liệu, các phương thức mock được gọi đúng tham số.</v>
@@ -3763,13 +3763,13 @@
     </row>
     <row r="4" xml:space="preserve">
       <c r="A4" t="str">
-        <v>STM-02</v>
+        <v>STM-01c</v>
       </c>
       <c r="B4" t="str">
-        <v>Khóa tài khoản không tồn tại ném lỗi 404</v>
+        <v>Mở khóa tài khoản học viên (isLocked = false)</v>
       </c>
       <c r="C4" t="str">
-        <v>Kiểm thử trường hợp biên &amp; Ngoại lệ (Negative / Bad Case)</v>
+        <v>Kiểm thử chức năng chuẩn (Happy Path)</v>
       </c>
       <c r="D4" t="str" xml:space="preserve">
         <v xml:space="preserve">1. Thiết lập Mock Repository / Database cho Service.
@@ -3777,21 +3777,21 @@
 3. Đối soát kết quả hoặc mã lỗi phát sinh.</v>
       </c>
       <c r="E4" t="str">
-        <v>Args: 9999, true</v>
+        <v>Args: 10, false</v>
       </c>
       <c r="F4" t="str">
-        <v>Ném ngoại lệ ApiError với status 404, mã lỗi 'ApiError'.</v>
+        <v>Hàm thực thi thành công, trả về đúng kiểu dữ liệu, các phương thức mock được gọi đúng tham số.</v>
       </c>
     </row>
     <row r="5" xml:space="preserve">
       <c r="A5" t="str">
-        <v>STM-03</v>
+        <v>STM-02a</v>
       </c>
       <c r="B5" t="str">
-        <v>Nhiều Admin cập nhật trạng thái khóa đồng thời</v>
+        <v>Khóa tài khoản không tồn tại ném lỗi 404</v>
       </c>
       <c r="C5" t="str">
-        <v>Kiểm thử đụng độ đồng thời (Concurrency / Race Condition)</v>
+        <v>Kiểm thử trường hợp biên &amp; Ngoại lệ (Negative / Bad Case)</v>
       </c>
       <c r="D5" t="str" xml:space="preserve">
         <v xml:space="preserve">1. Thiết lập Mock Repository / Database cho Service.
@@ -3799,147 +3799,609 @@
 3. Đối soát kết quả hoặc mã lỗi phát sinh.</v>
       </c>
       <c r="E5" t="str">
-        <v>Args: 10, false</v>
+        <v>Args: 9999, true</v>
       </c>
       <c r="F5" t="str">
-        <v>Hàm thực thi thành công, trả về đúng kiểu dữ liệu, các phương thức mock được gọi đúng tham số.</v>
+        <v>Ném ngoại lệ ApiError với status 404, mã lỗi 'student_not_found'.</v>
       </c>
     </row>
     <row r="6" xml:space="preserve">
       <c r="A6" t="str">
-        <v>STM-05</v>
+        <v>STM-02b</v>
       </c>
       <c r="B6" t="str">
-        <v>Mất kết nối DB khi truy vấn danh sách học viên ném lỗi 500</v>
+        <v>Lấy chi tiết học viên không tồn tại ném lỗi 404</v>
       </c>
       <c r="C6" t="str">
-        <v>Kiểm thử mất kết nối mạng &amp; Lỗi hệ thống (Network &amp; System Error)</v>
+        <v>Kiểm thử trường hợp biên &amp; Ngoại lệ (Negative / Bad Case)</v>
       </c>
       <c r="D6" t="str" xml:space="preserve">
         <v xml:space="preserve">1. Thiết lập Mock Repository / Database cho Service.
-2. Gọi method service.getStudentslist() với tham số kiểm thử.
+2. Gọi method service.getStudentDetail() với tham số kiểm thử.
 3. Đối soát kết quả hoặc mã lỗi phát sinh.</v>
       </c>
       <c r="E6" t="str">
-        <v>Args: { page: 1, limit: 10 }</v>
+        <v>Args: 9999</v>
       </c>
       <c r="F6" t="str">
-        <v>Ném ngoại lệ ApiError với status 4xx, mã lỗi 'ApiError'.</v>
+        <v>Ném ngoại lệ ApiError với status 404, mã lỗi 'student_not_found'.</v>
       </c>
     </row>
     <row r="7" xml:space="preserve">
       <c r="A7" t="str">
-        <v>STM-IT-01</v>
+        <v>STM-03a</v>
       </c>
       <c r="B7" t="str">
-        <v>GET /api/admin/students trả về danh sách học viên</v>
+        <v>Nhiều Admin cập nhật trạng thái khóa đồng thời</v>
       </c>
       <c r="C7" t="str">
-        <v>Kiểm thử chức năng chuẩn (Happy Path)</v>
+        <v>Kiểm thử đụng độ đồng thời (Concurrency / Race Condition - Update vs Delete)</v>
       </c>
       <c r="D7" t="str" xml:space="preserve">
-        <v xml:space="preserve">1. Thiết lập phiên đăng nhập / Mock quyền truy cập tương ứng.
-2. Gửi request HTTP GET tới endpoint /api/admin/students.
-3. Xác thực mã trạng thái HTTP và cấu trúc JSON trả về.</v>
+        <v xml:space="preserve">1. Thiết lập Mock Repository / Database cho Service.
+2. Gọi method service.updateStudentLockStatus() với tham số kiểm thử.
+3. Đối soát kết quả hoặc mã lỗi phát sinh.</v>
       </c>
       <c r="E7" t="str">
-        <v>Path param hoặc Payload chuẩn của StudentManage</v>
+        <v>Args: 10, false</v>
       </c>
       <c r="F7" t="str">
-        <v>HTTP Status: 200. Response trả về success = true cùng dữ liệu hợp lệ.</v>
+        <v>Hệ thống phân giải đụng độ an toàn: phát hiện bản ghi đã bị xóa (P2025/404) hoặc cập nhật nguyên tử, không sinh trạng thái zombie.</v>
       </c>
     </row>
     <row r="8" xml:space="preserve">
       <c r="A8" t="str">
-        <v>STM-IT-02</v>
+        <v>STM-03b</v>
       </c>
       <c r="B8" t="str">
-        <v>PATCH /api/admin/students/:id/status cập nhật trạng thái khóa tài khoản</v>
+        <v>Đụng độ Cập nhật &amp; Xóa: Admin cập nhật trạng thái khi tài khoản bị xóa đồng thời ném 404</v>
       </c>
       <c r="C8" t="str">
-        <v>Kiểm thử chức năng chuẩn (Happy Path)</v>
+        <v>Kiểm thử đụng độ đồng thời (Concurrency / Race Condition - Update vs Delete)</v>
       </c>
       <c r="D8" t="str" xml:space="preserve">
-        <v xml:space="preserve">1. Thiết lập phiên đăng nhập / Mock quyền truy cập tương ứng.
-2. Gửi request HTTP PATCH tới endpoint /api/admin/students/:id/status.
-3. Xác thực mã trạng thái HTTP và cấu trúc JSON trả về.</v>
+        <v xml:space="preserve">1. Thiết lập Mock Repository / Database cho Service.
+2. Gọi method service.updateStudentLockStatus() với tham số kiểm thử.
+3. Đối soát kết quả hoặc mã lỗi phát sinh.</v>
       </c>
       <c r="E8" t="str">
-        <v>Path param hoặc Payload chuẩn của StudentManage</v>
+        <v>Args: 10, true</v>
       </c>
       <c r="F8" t="str">
-        <v>HTTP Status: 200. Response trả về success = true cùng dữ liệu hợp lệ.</v>
+        <v>Ném ngoại lệ ApiError với status 4xx, mã lỗi 'ApiError'.</v>
       </c>
     </row>
     <row r="9" xml:space="preserve">
       <c r="A9" t="str">
-        <v>STM-IT-03</v>
+        <v>STM-03c</v>
       </c>
       <c r="B9" t="str">
-        <v>PATCH /api/admin/students/:id/status thiếu isLocked trả về 422</v>
+        <v>Đụng độ giữa Xem chi tiết và Xóa tài khoản: User bị xóa ngay khi đang truy vấn chi tiết</v>
       </c>
       <c r="C9" t="str">
-        <v>Kiểm thử trường hợp biên &amp; Ngoại lệ (Negative / Bad Case)</v>
+        <v>Kiểm thử đụng độ đồng thời (Concurrency / Race Condition - Update vs Delete)</v>
       </c>
       <c r="D9" t="str" xml:space="preserve">
-        <v xml:space="preserve">1. Thiết lập phiên đăng nhập / Mock quyền truy cập tương ứng.
-2. Gửi request HTTP PATCH tới endpoint /api/admin/students/:id/status.
-3. Xác thực mã trạng thái HTTP và cấu trúc JSON trả về.</v>
+        <v xml:space="preserve">1. Thiết lập Mock Repository / Database cho Service.
+2. Gọi method service.getStudentDetail() với tham số kiểm thử.
+3. Đối soát kết quả hoặc mã lỗi phát sinh.</v>
       </c>
       <c r="E9" t="str">
-        <v>{}</v>
+        <v>Args: 10</v>
       </c>
       <c r="F9" t="str">
-        <v>HTTP Status: 422. Báo lỗi validation hoặc bad request rõ ràng, không làm crash server.</v>
+        <v>Ném ngoại lệ ApiError với status 404, mã lỗi 'student_not_found'.</v>
       </c>
     </row>
     <row r="10" xml:space="preserve">
       <c r="A10" t="str">
-        <v>STM-IT-04</v>
+        <v>STM-03d</v>
       </c>
       <c r="B10" t="str">
-        <v>Gửi 2 request thay đổi trạng thái khóa học viên đồng thời</v>
+        <v>Đụng độ Cập nhật tới trước - Xóa xen ngang: Cập nhật không làm vô hiệu hóa việc xóa</v>
       </c>
       <c r="C10" t="str">
-        <v>Kiểm thử đụng độ đồng thời (Concurrency / Race Condition)</v>
+        <v>Kiểm thử đụng độ đồng thời (Concurrency / Race Condition - Update vs Delete)</v>
       </c>
       <c r="D10" t="str" xml:space="preserve">
-        <v xml:space="preserve">1. Thiết lập phiên đăng nhập / Mock quyền truy cập tương ứng.
-2. Gửi request HTTP PATCH tới endpoint /api/admin/students/10/status.
-3. Xác thực mã trạng thái HTTP và cấu trúc JSON trả về.</v>
+        <v xml:space="preserve">1. Thiết lập Mock Repository / Database cho Service.
+2. Gọi method service.updateStudentLockStatus() với tham số kiểm thử.
+3. Đối soát kết quả hoặc mã lỗi phát sinh.</v>
       </c>
       <c r="E10" t="str">
-        <v>{ isLocked: false }</v>
+        <v>Args: 10, true</v>
       </c>
       <c r="F10" t="str">
-        <v>HTTP Status: 200. Response trả về success = true cùng dữ liệu hợp lệ.</v>
+        <v>Ném ngoại lệ ApiError với status 4xx, mã lỗi 'ApiError'.</v>
       </c>
     </row>
     <row r="11" xml:space="preserve">
       <c r="A11" t="str">
+        <v>STM-04</v>
+      </c>
+      <c r="B11" t="str">
+        <v>Lỗi khi thu hồi refresh tokens khi khóa tài khoản ném ngoại lệ an toàn</v>
+      </c>
+      <c r="C11" t="str">
+        <v>Kiểm thử toàn vẹn dữ liệu &amp; Xung đột (Data Conflict / Rollback)</v>
+      </c>
+      <c r="D11" t="str" xml:space="preserve">
+        <v xml:space="preserve">1. Thiết lập Mock Repository / Database cho Service.
+2. Gọi method service.updateStudentLockStatus() với tham số kiểm thử.
+3. Đối soát kết quả hoặc mã lỗi phát sinh.</v>
+      </c>
+      <c r="E11" t="str">
+        <v>Args: 10, true</v>
+      </c>
+      <c r="F11" t="str">
+        <v>Ném ngoại lệ ApiError với status 4xx, mã lỗi 'ApiError'.</v>
+      </c>
+    </row>
+    <row r="12" xml:space="preserve">
+      <c r="A12" t="str">
+        <v>STM-05</v>
+      </c>
+      <c r="B12" t="str">
+        <v>Mất kết nối DB khi truy vấn danh sách học viên ném lỗi 500</v>
+      </c>
+      <c r="C12" t="str">
+        <v>Kiểm thử toàn vẹn dữ liệu &amp; Xung đột (Data Conflict / Rollback)</v>
+      </c>
+      <c r="D12" t="str" xml:space="preserve">
+        <v xml:space="preserve">1. Thiết lập Mock Repository / Database cho Service.
+2. Gọi method service.getStudentslist() với tham số kiểm thử.
+3. Đối soát kết quả hoặc mã lỗi phát sinh.</v>
+      </c>
+      <c r="E12" t="str">
+        <v>Args: { page: 1, limit: 10, sortBy: 'createdAt', sortOrder: 'desc', }</v>
+      </c>
+      <c r="F12" t="str">
+        <v>Ném ngoại lệ ApiError với status 4xx, mã lỗi 'ApiError'.</v>
+      </c>
+    </row>
+    <row r="13" xml:space="preserve">
+      <c r="A13" t="str">
+        <v>STM-AUTH-01</v>
+      </c>
+      <c r="B13" t="str">
+        <v>Chặn hành vi khóa tài khoản Admin: Không thể thao túng tài khoản có role khác</v>
+      </c>
+      <c r="C13" t="str">
+        <v>Kiểm thử phân quyền &amp; Bảo mật (Authorization &amp; Security 401/403)</v>
+      </c>
+      <c r="D13" t="str" xml:space="preserve">
+        <v xml:space="preserve">1. Thiết lập Mock Repository / Database cho Service.
+2. Gọi method service.updateStudentLockStatus() với tham số kiểm thử.
+3. Đối soát kết quả hoặc mã lỗi phát sinh.</v>
+      </c>
+      <c r="E13" t="str">
+        <v>Args: 99, true</v>
+      </c>
+      <c r="F13" t="str">
+        <v>Ném ngoại lệ ApiError với status 404, mã lỗi 'student_not_found'.</v>
+      </c>
+    </row>
+    <row r="14" xml:space="preserve">
+      <c r="A14" t="str">
+        <v>STM-AUTH-02</v>
+      </c>
+      <c r="B14" t="str">
+        <v>Đảm bảo kiểm tra nghiêm ngặt role học viên (role =</v>
+      </c>
+      <c r="C14" t="str">
+        <v>Kiểm thử phân quyền &amp; Bảo mật (Authorization &amp; Security 401/403)</v>
+      </c>
+      <c r="D14" t="str" xml:space="preserve">
+        <v xml:space="preserve">1. Thiết lập Mock Repository / Database cho Service.
+2. Gọi method service.updateStudentLockStatus() với tham số kiểm thử.
+3. Đối soát kết quả hoặc mã lỗi phát sinh.</v>
+      </c>
+      <c r="E14" t="str">
+        <v>Args: 1, false</v>
+      </c>
+      <c r="F14" t="str">
+        <v>Ném ngoại lệ ApiError với status 404, mã lỗi 'ApiError'.</v>
+      </c>
+    </row>
+    <row r="15" xml:space="preserve">
+      <c r="A15" t="str">
+        <v>STM-AUTH-03</v>
+      </c>
+      <c r="B15" t="str">
+        <v>Bảo mật phiên: Thu hồi tức thì toàn bộ Refresh Token khi tài khoản bị khóa</v>
+      </c>
+      <c r="C15" t="str">
+        <v>Kiểm thử phân quyền &amp; Bảo mật (Authorization &amp; Security 401/403)</v>
+      </c>
+      <c r="D15" t="str" xml:space="preserve">
+        <v xml:space="preserve">1. Thiết lập Mock Repository / Database cho Service.
+2. Gọi method service.updateStudentLockStatus() với tham số kiểm thử.
+3. Đối soát kết quả hoặc mã lỗi phát sinh.</v>
+      </c>
+      <c r="E15" t="str">
+        <v>Args: 10, true</v>
+      </c>
+      <c r="F15" t="str">
+        <v>Hàm thực thi thành công, trả về đúng kiểu dữ liệu, các phương thức mock được gọi đúng tham số.</v>
+      </c>
+    </row>
+    <row r="16" xml:space="preserve">
+      <c r="A16" t="str">
+        <v>STM-IT-AUTH-01</v>
+      </c>
+      <c r="B16" t="str">
+        <v>GET /api/admin/students: Học viên (role: user) truy cập danh sách bị chặn 403 Forbidden</v>
+      </c>
+      <c r="C16" t="str">
+        <v>Kiểm thử phân quyền &amp; Bảo mật (Authorization &amp; Security 401/403)</v>
+      </c>
+      <c r="D16" t="str" xml:space="preserve">
+        <v xml:space="preserve">1. Thiết lập phiên đăng nhập / Mock quyền truy cập tương ứng.
+2. Gửi request HTTP GET tới endpoint /api/admin/students.
+3. Xác thực mã trạng thái HTTP và cấu trúc JSON trả về.</v>
+      </c>
+      <c r="E16" t="str">
+        <v>Path param hoặc Payload chuẩn của StudentManage</v>
+      </c>
+      <c r="F16" t="str">
+        <v>HTTP Status: 403. Báo lỗi forbidden do tài khoản không có quyền truy cập thông tin quản trị.</v>
+      </c>
+    </row>
+    <row r="17" xml:space="preserve">
+      <c r="A17" t="str">
+        <v>STM-IT-AUTH-02</v>
+      </c>
+      <c r="B17" t="str">
+        <v>GET /api/admin/students/totalStudent: Học viên (role: user) xem tổng số học viên bị chặn 403 Forbidden</v>
+      </c>
+      <c r="C17" t="str">
+        <v>Kiểm thử phân quyền &amp; Bảo mật (Authorization &amp; Security 401/403)</v>
+      </c>
+      <c r="D17" t="str" xml:space="preserve">
+        <v xml:space="preserve">1. Thiết lập phiên đăng nhập / Mock quyền truy cập tương ứng.
+2. Gửi request HTTP GET tới endpoint /api/admin/students/totalStudent.
+3. Xác thực mã trạng thái HTTP và cấu trúc JSON trả về.</v>
+      </c>
+      <c r="E17" t="str">
+        <v>Path param hoặc Payload chuẩn của StudentManage</v>
+      </c>
+      <c r="F17" t="str">
+        <v>HTTP Status: 403. Báo lỗi forbidden do tài khoản không có quyền truy cập thông tin quản trị.</v>
+      </c>
+    </row>
+    <row r="18" xml:space="preserve">
+      <c r="A18" t="str">
+        <v>STM-IT-AUTH-03</v>
+      </c>
+      <c r="B18" t="str">
+        <v>GET /api/admin/students/top: Học viên (role: user) xem danh sách top học viên bị chặn 403 Forbidden</v>
+      </c>
+      <c r="C18" t="str">
+        <v>Kiểm thử phân quyền &amp; Bảo mật (Authorization &amp; Security 401/403)</v>
+      </c>
+      <c r="D18" t="str" xml:space="preserve">
+        <v xml:space="preserve">1. Thiết lập phiên đăng nhập / Mock quyền truy cập tương ứng.
+2. Gửi request HTTP GET tới endpoint /api/admin/students/top.
+3. Xác thực mã trạng thái HTTP và cấu trúc JSON trả về.</v>
+      </c>
+      <c r="E18" t="str">
+        <v>Path param hoặc Payload chuẩn của StudentManage</v>
+      </c>
+      <c r="F18" t="str">
+        <v>HTTP Status: 403. Báo lỗi forbidden do tài khoản không có quyền truy cập thông tin quản trị.</v>
+      </c>
+    </row>
+    <row r="19" xml:space="preserve">
+      <c r="A19" t="str">
+        <v>STM-IT-AUTH-04</v>
+      </c>
+      <c r="B19" t="str">
+        <v>GET /api/admin/students/:id: Học viên (role: user) xem chi tiết hồ sơ người khác bị chặn 403 Forbidden</v>
+      </c>
+      <c r="C19" t="str">
+        <v>Kiểm thử phân quyền &amp; Bảo mật (Authorization &amp; Security 401/403)</v>
+      </c>
+      <c r="D19" t="str" xml:space="preserve">
+        <v xml:space="preserve">1. Thiết lập phiên đăng nhập / Mock quyền truy cập tương ứng.
+2. Gửi request HTTP GET tới endpoint /api/admin/students/10.
+3. Xác thực mã trạng thái HTTP và cấu trúc JSON trả về.</v>
+      </c>
+      <c r="E19" t="str">
+        <v>Path param hoặc Payload chuẩn của StudentManage</v>
+      </c>
+      <c r="F19" t="str">
+        <v>HTTP Status: 403. Báo lỗi forbidden do tài khoản không có quyền truy cập thông tin quản trị.</v>
+      </c>
+    </row>
+    <row r="20" xml:space="preserve">
+      <c r="A20" t="str">
+        <v>STM-IT-AUTH-05</v>
+      </c>
+      <c r="B20" t="str">
+        <v>GET /api/admin/students/:id/progress: Học viên (role: user) xem tiến độ từ vựng người khác bị chặn 403 Forbidden</v>
+      </c>
+      <c r="C20" t="str">
+        <v>Kiểm thử phân quyền &amp; Bảo mật (Authorization &amp; Security 401/403)</v>
+      </c>
+      <c r="D20" t="str" xml:space="preserve">
+        <v xml:space="preserve">1. Thiết lập phiên đăng nhập / Mock quyền truy cập tương ứng.
+2. Gửi request HTTP GET tới endpoint /api/admin/students/10/progress.
+3. Xác thực mã trạng thái HTTP và cấu trúc JSON trả về.</v>
+      </c>
+      <c r="E20" t="str">
+        <v>Path param hoặc Payload chuẩn của StudentManage</v>
+      </c>
+      <c r="F20" t="str">
+        <v>HTTP Status: 403. Báo lỗi forbidden do tài khoản không có quyền truy cập thông tin quản trị.</v>
+      </c>
+    </row>
+    <row r="21" xml:space="preserve">
+      <c r="A21" t="str">
+        <v>STM-IT-AUTH-06</v>
+      </c>
+      <c r="B21" t="str">
+        <v>GET /api/admin/students/:id/ai-chat: Học viên (role: user) xem lịch sử chat AI người khác bị chặn 403 Forbidden</v>
+      </c>
+      <c r="C21" t="str">
+        <v>Kiểm thử phân quyền &amp; Bảo mật (Authorization &amp; Security 401/403)</v>
+      </c>
+      <c r="D21" t="str" xml:space="preserve">
+        <v xml:space="preserve">1. Thiết lập phiên đăng nhập / Mock quyền truy cập tương ứng.
+2. Gửi request HTTP GET tới endpoint /api/admin/students/10/ai-chat.
+3. Xác thực mã trạng thái HTTP và cấu trúc JSON trả về.</v>
+      </c>
+      <c r="E21" t="str">
+        <v>Path param hoặc Payload chuẩn của StudentManage</v>
+      </c>
+      <c r="F21" t="str">
+        <v>HTTP Status: 403. Báo lỗi forbidden do tài khoản không có quyền truy cập thông tin quản trị.</v>
+      </c>
+    </row>
+    <row r="22" xml:space="preserve">
+      <c r="A22" t="str">
+        <v>STM-IT-AUTH-07</v>
+      </c>
+      <c r="B22" t="str">
+        <v>PATCH /api/admin/students/:id/status: Học viên cố tình khóa tài khoản bị chặn 403 Forbidden</v>
+      </c>
+      <c r="C22" t="str">
+        <v>Kiểm thử phân quyền &amp; Bảo mật (Authorization &amp; Security 401/403)</v>
+      </c>
+      <c r="D22" t="str" xml:space="preserve">
+        <v xml:space="preserve">1. Thiết lập phiên đăng nhập / Mock quyền truy cập tương ứng.
+2. Gửi request HTTP PATCH tới endpoint /api/admin/students/:id/status:.
+3. Xác thực mã trạng thái HTTP và cấu trúc JSON trả về.</v>
+      </c>
+      <c r="E22" t="str">
+        <v>{ isLocked: true }</v>
+      </c>
+      <c r="F22" t="str">
+        <v>HTTP Status: 403. Báo lỗi forbidden do tài khoản không có quyền truy cập thông tin quản trị.</v>
+      </c>
+    </row>
+    <row r="23" xml:space="preserve">
+      <c r="A23" t="str">
+        <v>STM-IT-AUTH-08</v>
+      </c>
+      <c r="B23" t="str">
+        <v>GET /api/admin/students: Request không gửi Token xác thực trả về 401 Unauthorized</v>
+      </c>
+      <c r="C23" t="str">
+        <v>Kiểm thử phân quyền &amp; Bảo mật (Authorization &amp; Security 401/403)</v>
+      </c>
+      <c r="D23" t="str" xml:space="preserve">
+        <v xml:space="preserve">1. Thiết lập phiên đăng nhập / Mock quyền truy cập tương ứng.
+2. Gửi request HTTP GET tới endpoint /api/admin/students.
+3. Xác thực mã trạng thái HTTP và cấu trúc JSON trả về.</v>
+      </c>
+      <c r="E23" t="str">
+        <v>Path param hoặc Payload chuẩn của StudentManage</v>
+      </c>
+      <c r="F23" t="str">
+        <v>HTTP Status: 401. Báo lỗi unauthorized do chưa cung cấp token xác thực.</v>
+      </c>
+    </row>
+    <row r="24" xml:space="preserve">
+      <c r="A24" t="str">
+        <v>STM-IT-AUTH-09</v>
+      </c>
+      <c r="B24" t="str">
+        <v>PATCH /api/admin/students/:id/status: Request không gửi Token xác thực trả về 401 Unauthorized</v>
+      </c>
+      <c r="C24" t="str">
+        <v>Kiểm thử phân quyền &amp; Bảo mật (Authorization &amp; Security 401/403)</v>
+      </c>
+      <c r="D24" t="str" xml:space="preserve">
+        <v xml:space="preserve">1. Thiết lập phiên đăng nhập / Mock quyền truy cập tương ứng.
+2. Gửi request HTTP PATCH tới endpoint /api/admin/students/:id/status:.
+3. Xác thực mã trạng thái HTTP và cấu trúc JSON trả về.</v>
+      </c>
+      <c r="E24" t="str">
+        <v>{ isLocked: true }</v>
+      </c>
+      <c r="F24" t="str">
+        <v>HTTP Status: 401. Báo lỗi unauthorized do chưa cung cấp token xác thực.</v>
+      </c>
+    </row>
+    <row r="25" xml:space="preserve">
+      <c r="A25" t="str">
+        <v>STM-IT-01</v>
+      </c>
+      <c r="B25" t="str">
+        <v>GET /api/admin/students trả về danh sách học viên</v>
+      </c>
+      <c r="C25" t="str">
+        <v>Kiểm thử chức năng chuẩn (Happy Path)</v>
+      </c>
+      <c r="D25" t="str" xml:space="preserve">
+        <v xml:space="preserve">1. Thiết lập phiên đăng nhập / Mock quyền truy cập tương ứng.
+2. Gửi request HTTP GET tới endpoint /api/admin/students?page=1&amp;limit=10.
+3. Xác thực mã trạng thái HTTP và cấu trúc JSON trả về.</v>
+      </c>
+      <c r="E25" t="str">
+        <v>Query parameters: page=1&amp;limit=10</v>
+      </c>
+      <c r="F25" t="str">
+        <v>HTTP Status: 200. Response trả về success = true cùng dữ liệu hợp lệ.</v>
+      </c>
+    </row>
+    <row r="26" xml:space="preserve">
+      <c r="A26" t="str">
+        <v>STM-IT-02</v>
+      </c>
+      <c r="B26" t="str">
+        <v>PATCH /api/admin/students/:id/status cập nhật trạng thái khóa tài khoản</v>
+      </c>
+      <c r="C26" t="str">
+        <v>Kiểm thử chức năng chuẩn (Happy Path)</v>
+      </c>
+      <c r="D26" t="str" xml:space="preserve">
+        <v xml:space="preserve">1. Thiết lập phiên đăng nhập / Mock quyền truy cập tương ứng.
+2. Gửi request HTTP PATCH tới endpoint /api/admin/students/:id/status.
+3. Xác thực mã trạng thái HTTP và cấu trúc JSON trả về.</v>
+      </c>
+      <c r="E26" t="str">
+        <v>{ isLocked: true }</v>
+      </c>
+      <c r="F26" t="str">
+        <v>HTTP Status: 200. Response trả về success = true cùng dữ liệu hợp lệ.</v>
+      </c>
+    </row>
+    <row r="27" xml:space="preserve">
+      <c r="A27" t="str">
+        <v>STM-IT-03</v>
+      </c>
+      <c r="B27" t="str">
+        <v>PATCH /api/admin/students/:id/status thiếu isLocked trả về 422</v>
+      </c>
+      <c r="C27" t="str">
+        <v>Kiểm thử trường hợp biên &amp; Ngoại lệ (Negative / Bad Case)</v>
+      </c>
+      <c r="D27" t="str" xml:space="preserve">
+        <v xml:space="preserve">1. Thiết lập phiên đăng nhập / Mock quyền truy cập tương ứng.
+2. Gửi request HTTP PATCH tới endpoint /api/admin/students/:id/status.
+3. Xác thực mã trạng thái HTTP và cấu trúc JSON trả về.</v>
+      </c>
+      <c r="E27" t="str">
+        <v>{}</v>
+      </c>
+      <c r="F27" t="str">
+        <v>HTTP Status: 422. Báo lỗi validation hoặc bad request rõ ràng, không làm crash server.</v>
+      </c>
+    </row>
+    <row r="28" xml:space="preserve">
+      <c r="A28" t="str">
+        <v>STM-IT-04</v>
+      </c>
+      <c r="B28" t="str">
+        <v>GET /api/admin/students/abc id không phải số trả về 422</v>
+      </c>
+      <c r="C28" t="str">
+        <v>Kiểm thử trường hợp biên &amp; Ngoại lệ (Negative / Bad Case)</v>
+      </c>
+      <c r="D28" t="str" xml:space="preserve">
+        <v xml:space="preserve">1. Thiết lập phiên đăng nhập / Mock quyền truy cập tương ứng.
+2. Gửi request HTTP GET tới endpoint /api/admin/students/abc.
+3. Xác thực mã trạng thái HTTP và cấu trúc JSON trả về.</v>
+      </c>
+      <c r="E28" t="str">
+        <v>Path param hoặc Payload chuẩn của StudentManage</v>
+      </c>
+      <c r="F28" t="str">
+        <v>HTTP Status: 422. Báo lỗi validation hoặc bad request rõ ràng, không làm crash server.</v>
+      </c>
+    </row>
+    <row r="29" xml:space="preserve">
+      <c r="A29" t="str">
+        <v>STM-IT-RACE-01</v>
+      </c>
+      <c r="B29" t="str">
+        <v>Đụng độ Cập nhật &amp; Xóa đồng thời: 1 request thành công, 1 request gặp tài khoản đã xóa trả về 404</v>
+      </c>
+      <c r="C29" t="str">
+        <v>Kiểm thử đụng độ đồng thời (Concurrency / Race Condition - Update vs Delete)</v>
+      </c>
+      <c r="D29" t="str" xml:space="preserve">
+        <v xml:space="preserve">1. Thiết lập phiên đăng nhập / Mock quyền truy cập tương ứng.
+2. Gửi request HTTP PATCH tới endpoint /api/admin/students/10/status.
+3. Xác thực mã trạng thái HTTP và cấu trúc JSON trả về.</v>
+      </c>
+      <c r="E29" t="str">
+        <v>{ isLocked: true }</v>
+      </c>
+      <c r="F29" t="str">
+        <v>HTTP Status: 200. Response trả về success = true cùng dữ liệu hợp lệ.</v>
+      </c>
+    </row>
+    <row r="30" xml:space="preserve">
+      <c r="A30" t="str">
+        <v>STM-IT-RACE-02</v>
+      </c>
+      <c r="B30" t="str">
+        <v>Gửi 2 request thay đổi trạng thái khóa học viên đồng thời</v>
+      </c>
+      <c r="C30" t="str">
+        <v>Kiểm thử đụng độ đồng thời (Concurrency / Race Condition - Update vs Delete)</v>
+      </c>
+      <c r="D30" t="str" xml:space="preserve">
+        <v xml:space="preserve">1. Thiết lập phiên đăng nhập / Mock quyền truy cập tương ứng.
+2. Gửi request HTTP PATCH tới endpoint /api/admin/students/10/status.
+3. Xác thực mã trạng thái HTTP và cấu trúc JSON trả về.</v>
+      </c>
+      <c r="E30" t="str">
+        <v>{ isLocked: false }</v>
+      </c>
+      <c r="F30" t="str">
+        <v>HTTP Status: 200. Response trả về success = true cùng dữ liệu hợp lệ.</v>
+      </c>
+    </row>
+    <row r="31" xml:space="preserve">
+      <c r="A31" t="str">
+        <v>STM-IT-RACE-03</v>
+      </c>
+      <c r="B31" t="str">
+        <v>Đụng độ Update tới trước - Delete xen ngang: Cập nhật không làm vô hiệu hóa kết quả xóa</v>
+      </c>
+      <c r="C31" t="str">
+        <v>Kiểm thử đụng độ đồng thời (Concurrency / Race Condition - Update vs Delete)</v>
+      </c>
+      <c r="D31" t="str" xml:space="preserve">
+        <v xml:space="preserve">1. Thiết lập phiên đăng nhập / Mock quyền truy cập tương ứng.
+2. Gửi request HTTP PATCH tới endpoint /api/admin/students/10/status.
+3. Xác thực mã trạng thái HTTP và cấu trúc JSON trả về.</v>
+      </c>
+      <c r="E31" t="str">
+        <v>{ isLocked: true }</v>
+      </c>
+      <c r="F31" t="str">
+        <v>HTTP Status: 404. Báo lỗi student_not_found do bản ghi đã bị xóa hoặc không tồn tại.</v>
+      </c>
+    </row>
+    <row r="32" xml:space="preserve">
+      <c r="A32" t="str">
         <v>STM-IT-05</v>
       </c>
-      <c r="B11" t="str">
+      <c r="B32" t="str">
         <v>Mất kết nối DB khi lấy danh sách học viên trả về 500</v>
       </c>
-      <c r="C11" t="str">
-        <v>Kiểm thử mất kết nối mạng &amp; Lỗi hệ thống (Network &amp; System Error)</v>
-      </c>
-      <c r="D11" t="str" xml:space="preserve">
+      <c r="C32" t="str">
+        <v>Kiểm thử toàn vẹn dữ liệu &amp; Xung đột (Data Conflict / Rollback)</v>
+      </c>
+      <c r="D32" t="str" xml:space="preserve">
         <v xml:space="preserve">1. Thiết lập phiên đăng nhập / Mock quyền truy cập tương ứng.
 2. Gửi request HTTP GET tới endpoint /api/admin/students?page=1&amp;limit=10.
 3. Xác thực mã trạng thái HTTP và cấu trúc JSON trả về.</v>
       </c>
-      <c r="E11" t="str">
+      <c r="E32" t="str">
         <v>Query parameters: page=1&amp;limit=10</v>
       </c>
-      <c r="F11" t="str">
+      <c r="F32" t="str">
         <v>HTTP Status: 500. Hệ thống bắt lỗi thông qua error-handler, trả về HTTP 500 an toàn.</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:F11"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:F32"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -3948,12 +4410,12 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:F18"/>
   <cols>
-    <col min="1" max="1" width="15.83203125" customWidth="1"/>
-    <col min="2" max="2" width="45.83203125" customWidth="1"/>
-    <col min="3" max="3" width="35.83203125" customWidth="1"/>
+    <col min="1" max="1" width="18.83203125" customWidth="1"/>
+    <col min="2" max="2" width="48.83203125" customWidth="1"/>
+    <col min="3" max="3" width="40.83203125" customWidth="1"/>
     <col min="4" max="4" width="45.83203125" customWidth="1"/>
     <col min="5" max="5" width="35.83203125" customWidth="1"/>
-    <col min="6" max="6" width="45.83203125" customWidth="1"/>
+    <col min="6" max="6" width="48.83203125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -3987,12 +4449,12 @@
         <v>Kiểm thử chức năng chuẩn (Happy Path)</v>
       </c>
       <c r="D2" t="str" xml:space="preserve">
-        <v xml:space="preserve">1. Khởi tạo Service với Mock Repository / Prisma Client.
-2. Kích hoạt hàm nghiệp vụ tương ứng của student-vocabulary.
-3. Kiểm tra giá trị trả về hoặc bắt exception.</v>
+        <v xml:space="preserve">1. Thiết lập Mock Repository / Database cho Service.
+2. Gọi method service.getVocabularyList() với tham số kiểm thử.
+3. Đối soát kết quả hoặc mã lỗi phát sinh.</v>
       </c>
       <c r="E2" t="str">
-        <v>Dữ liệu test fixture trong student-vocabulary.mock.ts</v>
+        <v>Args: 1, { limit: 10 }</v>
       </c>
       <c r="F2" t="str">
         <v>Hàm thực thi thành công, trả về đúng kiểu dữ liệu, các phương thức mock được gọi đúng tham số.</v>
@@ -4014,7 +4476,7 @@
 3. Đối soát kết quả hoặc mã lỗi phát sinh.</v>
       </c>
       <c r="E3" t="str">
-        <v>Args: 1, { wordId: 10 }</v>
+        <v>Args: 1, { wordId: 10, status: 'new' }</v>
       </c>
       <c r="F3" t="str">
         <v>Hàm thực thi thành công, trả về đúng kiểu dữ liệu, các phương thức mock được gọi đúng tham số.</v>
@@ -4102,7 +4564,7 @@
 3. Đối soát kết quả hoặc mã lỗi phát sinh.</v>
       </c>
       <c r="E7" t="str">
-        <v>Args: 1, { wordId: 999 }</v>
+        <v>Args: 1, { wordId: 999, status: 'new' }</v>
       </c>
       <c r="F7" t="str">
         <v>Ném ngoại lệ ApiError với status 404, mã lỗi 'ApiError'.</v>
@@ -4116,7 +4578,7 @@
         <v>Nộp ôn tập song song nhiều từ vựng được thực thi an toàn</v>
       </c>
       <c r="C8" t="str">
-        <v>Kiểm thử đụng độ đồng thời (Concurrency / Race Condition)</v>
+        <v>Kiểm thử đụng độ đồng thời (Concurrency / Race Condition - Update vs Delete)</v>
       </c>
       <c r="D8" t="str" xml:space="preserve">
         <v xml:space="preserve">1. Thiết lập Mock Repository / Database cho Service.
@@ -4127,7 +4589,7 @@
         <v>Args: 1, 10, true</v>
       </c>
       <c r="F8" t="str">
-        <v>Hàm thực thi thành công, trả về đúng kiểu dữ liệu, các phương thức mock được gọi đúng tham số.</v>
+        <v>Hệ thống phân giải đụng độ an toàn: phát hiện bản ghi đã bị xóa (P2025/404) hoặc cập nhật nguyên tử, không sinh trạng thái zombie.</v>
       </c>
     </row>
     <row r="9" xml:space="preserve">
@@ -4138,7 +4600,7 @@
         <v>Chặn thêm từ vựng đã có sẵn trong danh sách của học viên (409 word_already_added)</v>
       </c>
       <c r="C9" t="str">
-        <v>Kiểm thử toàn vẹn dữ liệu &amp; Xung đột (Data Conflict / Rollback)</v>
+        <v>Kiểm thử phân quyền &amp; Bảo mật (Authorization &amp; Security 401/403)</v>
       </c>
       <c r="D9" t="str" xml:space="preserve">
         <v xml:space="preserve">1. Thiết lập Mock Repository / Database cho Service.
@@ -4146,7 +4608,7 @@
 3. Đối soát kết quả hoặc mã lỗi phát sinh.</v>
       </c>
       <c r="E9" t="str">
-        <v>Args: 1, { wordId: 10 }</v>
+        <v>Args: 1, { wordId: 10, status: 'new' }</v>
       </c>
       <c r="F9" t="str">
         <v>Ném ngoại lệ ApiError với status 409, mã lỗi 'word_already_added'.</v>
@@ -4160,7 +4622,7 @@
         <v>Mất kết nối DB khi nộp ôn tập rollback transaction sạch sẽ</v>
       </c>
       <c r="C10" t="str">
-        <v>Kiểm thử mất kết nối mạng &amp; Lỗi hệ thống (Network &amp; System Error)</v>
+        <v>Kiểm thử toàn vẹn dữ liệu &amp; Xung đột (Data Conflict / Rollback)</v>
       </c>
       <c r="D10" t="str" xml:space="preserve">
         <v xml:space="preserve">1. Thiết lập Mock Repository / Database cho Service.
@@ -4281,7 +4743,7 @@
         <v>Path param hoặc Payload chuẩn của student-vocabulary</v>
       </c>
       <c r="F15" t="str">
-        <v xml:space="preserve">HTTP Status: 404. </v>
+        <v>HTTP Status: 404. Báo lỗi student_not_found do bản ghi đã bị xóa hoặc không tồn tại.</v>
       </c>
     </row>
     <row r="16" xml:space="preserve">
@@ -4292,7 +4754,7 @@
         <v>Gửi 2 request ôn tập song song</v>
       </c>
       <c r="C16" t="str">
-        <v>Kiểm thử đụng độ đồng thời (Concurrency / Race Condition)</v>
+        <v>Kiểm thử đụng độ đồng thời (Concurrency / Race Condition - Update vs Delete)</v>
       </c>
       <c r="D16" t="str" xml:space="preserve">
         <v xml:space="preserve">1. Thiết lập phiên đăng nhập / Mock quyền truy cập tương ứng.
@@ -4314,7 +4776,7 @@
         <v>Thêm từ đã có sẵn trả về 409 Conflict</v>
       </c>
       <c r="C17" t="str">
-        <v>Kiểm thử mất kết nối mạng &amp; Lỗi hệ thống (Network &amp; System Error)</v>
+        <v>Kiểm thử toàn vẹn dữ liệu &amp; Xung đột (Data Conflict / Rollback)</v>
       </c>
       <c r="D17" t="str" xml:space="preserve">
         <v xml:space="preserve">1. Thiết lập phiên đăng nhập / Mock quyền truy cập tương ứng.
@@ -4336,7 +4798,7 @@
         <v>Mất kết nối DB khi lấy danh sách trả về 500</v>
       </c>
       <c r="C18" t="str">
-        <v>Kiểm thử mất kết nối mạng &amp; Lỗi hệ thống (Network &amp; System Error)</v>
+        <v>Kiểm thử toàn vẹn dữ liệu &amp; Xung đột (Data Conflict / Rollback)</v>
       </c>
       <c r="D18" t="str" xml:space="preserve">
         <v xml:space="preserve">1. Thiết lập phiên đăng nhập / Mock quyền truy cập tương ứng.
@@ -4361,12 +4823,12 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:F18"/>
   <cols>
-    <col min="1" max="1" width="15.83203125" customWidth="1"/>
-    <col min="2" max="2" width="45.83203125" customWidth="1"/>
-    <col min="3" max="3" width="35.83203125" customWidth="1"/>
+    <col min="1" max="1" width="18.83203125" customWidth="1"/>
+    <col min="2" max="2" width="48.83203125" customWidth="1"/>
+    <col min="3" max="3" width="40.83203125" customWidth="1"/>
     <col min="4" max="4" width="45.83203125" customWidth="1"/>
     <col min="5" max="5" width="35.83203125" customWidth="1"/>
-    <col min="6" max="6" width="45.83203125" customWidth="1"/>
+    <col min="6" max="6" width="48.83203125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -4444,12 +4906,12 @@
         <v>Kiểm thử chức năng chuẩn (Happy Path)</v>
       </c>
       <c r="D4" t="str" xml:space="preserve">
-        <v xml:space="preserve">1. Khởi tạo Service với Mock Repository / Prisma Client.
-2. Kích hoạt hàm nghiệp vụ tương ứng của test.
-3. Kiểm tra giá trị trả về hoặc bắt exception.</v>
+        <v xml:space="preserve">1. Thiết lập Mock Repository / Database cho Service.
+2. Gọi method service.addQuestion() với tham số kiểm thử.
+3. Đối soát kết quả hoặc mã lỗi phát sinh.</v>
       </c>
       <c r="E4" t="str">
-        <v>Dữ liệu test fixture trong test.mock.ts</v>
+        <v>Args: 1, mockCreateQuestionInput</v>
       </c>
       <c r="F4" t="str">
         <v>Hàm thực thi thành công, trả về đúng kiểu dữ liệu, các phương thức mock được gọi đúng tham số.</v>
@@ -4551,7 +5013,7 @@
         <v>Hai yêu cầu xóa bài thi cùng lúc xử lý an toàn</v>
       </c>
       <c r="C9" t="str">
-        <v>Kiểm thử đụng độ đồng thời (Concurrency / Race Condition)</v>
+        <v>Kiểm thử đụng độ đồng thời (Concurrency / Race Condition - Update vs Delete)</v>
       </c>
       <c r="D9" t="str" xml:space="preserve">
         <v xml:space="preserve">1. Thiết lập Mock Repository / Database cho Service.
@@ -4573,7 +5035,7 @@
         <v>Mất kết nối DB khi lấy danh sách câu hỏi ném lỗi hệ thống</v>
       </c>
       <c r="C10" t="str">
-        <v>Kiểm thử mất kết nối mạng &amp; Lỗi hệ thống (Network &amp; System Error)</v>
+        <v>Kiểm thử toàn vẹn dữ liệu &amp; Xung đột (Data Conflict / Rollback)</v>
       </c>
       <c r="D10" t="str" xml:space="preserve">
         <v xml:space="preserve">1. Thiết lập Mock Repository / Database cho Service.
@@ -4595,7 +5057,7 @@
         <v>Lỗi Rollback transaction khi lưu câu hỏi và đáp án ném lỗi</v>
       </c>
       <c r="C11" t="str">
-        <v>Kiểm thử mất kết nối mạng &amp; Lỗi hệ thống (Network &amp; System Error)</v>
+        <v>Kiểm thử toàn vẹn dữ liệu &amp; Xung đột (Data Conflict / Rollback)</v>
       </c>
       <c r="D11" t="str" xml:space="preserve">
         <v xml:space="preserve">1. Thiết lập Mock Repository / Database cho Service.
@@ -4774,12 +5236,12 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:F12"/>
   <cols>
-    <col min="1" max="1" width="15.83203125" customWidth="1"/>
-    <col min="2" max="2" width="45.83203125" customWidth="1"/>
-    <col min="3" max="3" width="35.83203125" customWidth="1"/>
+    <col min="1" max="1" width="18.83203125" customWidth="1"/>
+    <col min="2" max="2" width="48.83203125" customWidth="1"/>
+    <col min="3" max="3" width="40.83203125" customWidth="1"/>
     <col min="4" max="4" width="45.83203125" customWidth="1"/>
     <col min="5" max="5" width="35.83203125" customWidth="1"/>
-    <col min="6" max="6" width="45.83203125" customWidth="1"/>
+    <col min="6" max="6" width="48.83203125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -4898,7 +5360,7 @@
         <v>Nhiều request sửa topic đồng thời</v>
       </c>
       <c r="C6" t="str">
-        <v>Kiểm thử đụng độ đồng thời (Concurrency / Race Condition)</v>
+        <v>Kiểm thử đụng độ đồng thời (Concurrency / Race Condition - Update vs Delete)</v>
       </c>
       <c r="D6" t="str" xml:space="preserve">
         <v xml:space="preserve">1. Thiết lập Mock Repository / Database cho Service.
@@ -4909,7 +5371,7 @@
         <v>Args: 1, { title: 'T1' }</v>
       </c>
       <c r="F6" t="str">
-        <v>Hàm thực thi thành công, trả về đúng kiểu dữ liệu, các phương thức mock được gọi đúng tham số.</v>
+        <v>Hệ thống phân giải đụng độ an toàn: phát hiện bản ghi đã bị xóa (P2025/404) hoặc cập nhật nguyên tử, không sinh trạng thái zombie.</v>
       </c>
     </row>
     <row r="7" xml:space="preserve">
@@ -4920,7 +5382,7 @@
         <v>Mất kết nối DB khi xóa topic ném lỗi hệ thống</v>
       </c>
       <c r="C7" t="str">
-        <v>Kiểm thử mất kết nối mạng &amp; Lỗi hệ thống (Network &amp; System Error)</v>
+        <v>Kiểm thử toàn vẹn dữ liệu &amp; Xung đột (Data Conflict / Rollback)</v>
       </c>
       <c r="D7" t="str" xml:space="preserve">
         <v xml:space="preserve">1. Thiết lập Mock Repository / Database cho Service.
@@ -5055,12 +5517,12 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:F10"/>
   <cols>
-    <col min="1" max="1" width="15.83203125" customWidth="1"/>
-    <col min="2" max="2" width="45.83203125" customWidth="1"/>
-    <col min="3" max="3" width="35.83203125" customWidth="1"/>
+    <col min="1" max="1" width="18.83203125" customWidth="1"/>
+    <col min="2" max="2" width="48.83203125" customWidth="1"/>
+    <col min="3" max="3" width="40.83203125" customWidth="1"/>
     <col min="4" max="4" width="45.83203125" customWidth="1"/>
     <col min="5" max="5" width="35.83203125" customWidth="1"/>
-    <col min="6" max="6" width="45.83203125" customWidth="1"/>
+    <col min="6" max="6" width="48.83203125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -5157,7 +5619,7 @@
         <v>Nhiều Admin cập nhật từ vựng song song</v>
       </c>
       <c r="C5" t="str">
-        <v>Kiểm thử đụng độ đồng thời (Concurrency / Race Condition)</v>
+        <v>Kiểm thử đụng độ đồng thời (Concurrency / Race Condition - Update vs Delete)</v>
       </c>
       <c r="D5" t="str" xml:space="preserve">
         <v xml:space="preserve">1. Khởi tạo Service với Mock Repository / Prisma Client.
@@ -5168,7 +5630,7 @@
         <v>Dữ liệu test fixture trong word.mock.ts</v>
       </c>
       <c r="F5" t="str">
-        <v>Hàm thực thi thành công, trả về đúng kiểu dữ liệu, các phương thức mock được gọi đúng tham số.</v>
+        <v>Hệ thống phân giải đụng độ an toàn: phát hiện bản ghi đã bị xóa (P2025/404) hoặc cập nhật nguyên tử, không sinh trạng thái zombie.</v>
       </c>
     </row>
     <row r="6" xml:space="preserve">
@@ -5179,7 +5641,7 @@
         <v>Mất kết nối DB khi xóa từ ném lỗi hệ thống</v>
       </c>
       <c r="C6" t="str">
-        <v>Kiểm thử mất kết nối mạng &amp; Lỗi hệ thống (Network &amp; System Error)</v>
+        <v>Kiểm thử toàn vẹn dữ liệu &amp; Xung đột (Data Conflict / Rollback)</v>
       </c>
       <c r="D6" t="str" xml:space="preserve">
         <v xml:space="preserve">1. Khởi tạo Service với Mock Repository / Prisma Client.
@@ -5292,12 +5754,12 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:F14"/>
   <cols>
-    <col min="1" max="1" width="15.83203125" customWidth="1"/>
-    <col min="2" max="2" width="45.83203125" customWidth="1"/>
-    <col min="3" max="3" width="35.83203125" customWidth="1"/>
+    <col min="1" max="1" width="18.83203125" customWidth="1"/>
+    <col min="2" max="2" width="48.83203125" customWidth="1"/>
+    <col min="3" max="3" width="40.83203125" customWidth="1"/>
     <col min="4" max="4" width="45.83203125" customWidth="1"/>
     <col min="5" max="5" width="35.83203125" customWidth="1"/>
-    <col min="6" max="6" width="45.83203125" customWidth="1"/>
+    <col min="6" max="6" width="48.83203125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -5438,7 +5900,7 @@
         <v>Hai yêu cầu nộp bài submit song song</v>
       </c>
       <c r="C7" t="str">
-        <v>Kiểm thử mất kết nối mạng &amp; Lỗi hệ thống (Network &amp; System Error)</v>
+        <v>Kiểm thử đụng độ đồng thời (Concurrency / Race Condition - Update vs Delete)</v>
       </c>
       <c r="D7" t="str" xml:space="preserve">
         <v xml:space="preserve">1. Thiết lập Mock Repository / Database cho Service.
@@ -5449,7 +5911,7 @@
         <v>Args: 1, mockSubmitWordMatchingInput</v>
       </c>
       <c r="F7" t="str">
-        <v>Ném ngoại lệ lỗi kết nối hoặc Rollback Transaction, không lưu dữ liệu rác.</v>
+        <v>Hệ thống phân giải đụng độ an toàn: phát hiện bản ghi đã bị xóa (P2025/404) hoặc cập nhật nguyên tử, không sinh trạng thái zombie.</v>
       </c>
     </row>
     <row r="8" xml:space="preserve">
@@ -5460,7 +5922,7 @@
         <v>Mất kết nối database khi nộp bài ném lỗi</v>
       </c>
       <c r="C8" t="str">
-        <v>Kiểm thử mất kết nối mạng &amp; Lỗi hệ thống (Network &amp; System Error)</v>
+        <v>Kiểm thử đụng độ đồng thời (Concurrency / Race Condition - Update vs Delete)</v>
       </c>
       <c r="D8" t="str" xml:space="preserve">
         <v xml:space="preserve">1. Thiết lập Mock Repository / Database cho Service.
@@ -5486,11 +5948,11 @@
       </c>
       <c r="D9" t="str" xml:space="preserve">
         <v xml:space="preserve">1. Thiết lập phiên đăng nhập / Mock quyền truy cập tương ứng.
-2. Gửi request HTTP GET tới endpoint /api/word-matching/start.
+2. Gửi request HTTP GET tới endpoint /api/word-matching/start?limit=4.
 3. Xác thực mã trạng thái HTTP và cấu trúc JSON trả về.</v>
       </c>
       <c r="E9" t="str">
-        <v>Path param hoặc Payload chuẩn của word-matching</v>
+        <v>Query parameters: limit=4</v>
       </c>
       <c r="F9" t="str">
         <v>HTTP Status: 200. Response trả về success = true cùng dữ liệu hợp lệ.</v>
@@ -5512,7 +5974,7 @@
 3. Xác thực mã trạng thái HTTP và cấu trúc JSON trả về.</v>
       </c>
       <c r="E10" t="str">
-        <v>Path param hoặc Payload chuẩn của word-matching</v>
+        <v>mockSubmitWordMatchingInput</v>
       </c>
       <c r="F10" t="str">
         <v>HTTP Status: 200. Response trả về success = true cùng dữ liệu hợp lệ.</v>
@@ -5534,7 +5996,7 @@
 3. Xác thực mã trạng thái HTTP và cấu trúc JSON trả về.</v>
       </c>
       <c r="E11" t="str">
-        <v>Path param hoặc Payload chuẩn của word-matching</v>
+        <v>mockSaveWordMatchingProgressInput</v>
       </c>
       <c r="F11" t="str">
         <v>HTTP Status: 200. Response trả về success = true cùng dữ liệu hợp lệ.</v>
@@ -5592,7 +6054,7 @@
         <v>Lỗi database khi nộp bài trả về 500</v>
       </c>
       <c r="C14" t="str">
-        <v>Kiểm thử mất kết nối mạng &amp; Lỗi hệ thống (Network &amp; System Error)</v>
+        <v>Kiểm thử trường hợp biên &amp; Ngoại lệ (Negative / Bad Case)</v>
       </c>
       <c r="D14" t="str" xml:space="preserve">
         <v xml:space="preserve">1. Thiết lập phiên đăng nhập / Mock quyền truy cập tương ứng.
@@ -5615,14 +6077,14 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F13"/>
+  <dimension ref="A1:F26"/>
   <cols>
-    <col min="1" max="1" width="15.83203125" customWidth="1"/>
-    <col min="2" max="2" width="45.83203125" customWidth="1"/>
-    <col min="3" max="3" width="35.83203125" customWidth="1"/>
+    <col min="1" max="1" width="18.83203125" customWidth="1"/>
+    <col min="2" max="2" width="48.83203125" customWidth="1"/>
+    <col min="3" max="3" width="40.83203125" customWidth="1"/>
     <col min="4" max="4" width="45.83203125" customWidth="1"/>
     <col min="5" max="5" width="35.83203125" customWidth="1"/>
-    <col min="6" max="6" width="45.83203125" customWidth="1"/>
+    <col min="6" max="6" width="48.83203125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -5735,13 +6197,13 @@
     </row>
     <row r="6" xml:space="preserve">
       <c r="A6" t="str">
-        <v>ACH-03</v>
+        <v>ACH-03a</v>
       </c>
       <c r="B6" t="str">
-        <v>Không mở khóa trùng lặp danh hiệu học viên đã sở hữu</v>
+        <v>Không mở khóa trùng lặp danh hiệu học viên đã sở hữu (Idempotency)</v>
       </c>
       <c r="C6" t="str">
-        <v>Kiểm thử toàn vẹn dữ liệu &amp; Xung đột (Data Conflict / Rollback)</v>
+        <v>Kiểm thử đụng độ đồng thời (Concurrency / Race Condition - Update vs Delete)</v>
       </c>
       <c r="D6" t="str" xml:space="preserve">
         <v xml:space="preserve">1. Khởi tạo Service với Mock Repository / Prisma Client.
@@ -5752,18 +6214,18 @@
         <v>Dữ liệu test fixture trong achievement.mock.ts</v>
       </c>
       <c r="F6" t="str">
-        <v>Hàm thực thi thành công, trả về đúng kiểu dữ liệu, các phương thức mock được gọi đúng tham số.</v>
+        <v>Hệ thống phân giải đụng độ an toàn: phát hiện bản ghi đã bị xóa (P2025/404) hoặc cập nhật nguyên tử, không sinh trạng thái zombie.</v>
       </c>
     </row>
     <row r="7" xml:space="preserve">
       <c r="A7" t="str">
-        <v>ACH-05</v>
+        <v>ACH-03b</v>
       </c>
       <c r="B7" t="str">
-        <v>Mất kết nối DB khi đánh giá danh hiệu không làm chết ứng dụng</v>
+        <v>Đánh giá mở khóa liên tiếp/đồng thời: Lần gọi thứ 2 phát hiện đã mở khóa sẽ bỏ qua</v>
       </c>
       <c r="C7" t="str">
-        <v>Kiểm thử mất kết nối mạng &amp; Lỗi hệ thống (Network &amp; System Error)</v>
+        <v>Kiểm thử đụng độ đồng thời (Concurrency / Race Condition - Update vs Delete)</v>
       </c>
       <c r="D7" t="str" xml:space="preserve">
         <v xml:space="preserve">1. Khởi tạo Service với Mock Repository / Prisma Client.
@@ -5774,158 +6236,444 @@
         <v>Dữ liệu test fixture trong achievement.mock.ts</v>
       </c>
       <c r="F7" t="str">
-        <v>Ném ngoại lệ ApiError với status 4xx, mã lỗi 'ApiError'.</v>
+        <v>Hệ thống phân giải đụng độ an toàn: phát hiện bản ghi đã bị xóa (P2025/404) hoặc cập nhật nguyên tử, không sinh trạng thái zombie.</v>
       </c>
     </row>
     <row r="8" xml:space="preserve">
       <c r="A8" t="str">
-        <v>ACH-IT-01</v>
+        <v>ACH-03c</v>
       </c>
       <c r="B8" t="str">
-        <v>GET /api/admin/achievements trả về danh sách danh hiệu</v>
+        <v>Đụng độ Cập nhật &amp; Xóa danh hiệu tại Service: Request update gặp record đã bị xóa ném 404</v>
       </c>
       <c r="C8" t="str">
-        <v>Kiểm thử chức năng chuẩn (Happy Path)</v>
+        <v>Kiểm thử đụng độ đồng thời (Concurrency / Race Condition - Update vs Delete)</v>
       </c>
       <c r="D8" t="str" xml:space="preserve">
-        <v xml:space="preserve">1. Thiết lập phiên đăng nhập / Mock quyền truy cập tương ứng.
-2. Gửi request HTTP GET tới endpoint /api/admin/achievements.
-3. Xác thực mã trạng thái HTTP và cấu trúc JSON trả về.</v>
+        <v xml:space="preserve">1. Thiết lập Mock Repository / Database cho Service.
+2. Gọi method service.update() với tham số kiểm thử.
+3. Đối soát kết quả hoặc mã lỗi phát sinh.</v>
       </c>
       <c r="E8" t="str">
-        <v>Path param hoặc Payload chuẩn của achievement</v>
+        <v>Args: 1, { title: 'Updated' }, 1</v>
       </c>
       <c r="F8" t="str">
-        <v>HTTP Status: 200. Response trả về success = true cùng dữ liệu hợp lệ.</v>
+        <v>Ném ngoại lệ ApiError với status 404, mã lỗi 'ApiError'.</v>
       </c>
     </row>
     <row r="9" xml:space="preserve">
       <c r="A9" t="str">
-        <v>ACH-IT-02</v>
+        <v>ACH-05</v>
       </c>
       <c r="B9" t="str">
-        <v>POST /api/admin/achievements tạo danh hiệu mới</v>
+        <v>Mất kết nối DB khi đánh giá danh hiệu không làm chết ứng dụng</v>
       </c>
       <c r="C9" t="str">
-        <v>Kiểm thử chức năng chuẩn (Happy Path)</v>
+        <v>Kiểm thử toàn vẹn dữ liệu &amp; Xung đột (Data Conflict / Rollback)</v>
       </c>
       <c r="D9" t="str" xml:space="preserve">
-        <v xml:space="preserve">1. Thiết lập phiên đăng nhập / Mock quyền truy cập tương ứng.
-2. Gửi request HTTP POST tới endpoint /api/admin/achievements.
-3. Xác thực mã trạng thái HTTP và cấu trúc JSON trả về.</v>
+        <v xml:space="preserve">1. Khởi tạo Service với Mock Repository / Prisma Client.
+2. Kích hoạt hàm nghiệp vụ tương ứng của achievement.
+3. Kiểm tra giá trị trả về hoặc bắt exception.</v>
       </c>
       <c r="E9" t="str">
-        <v>{ title: 'Bậc thầy', requireXp: 1000, requireStreak: 30 }</v>
+        <v>Dữ liệu test fixture trong achievement.mock.ts</v>
       </c>
       <c r="F9" t="str">
-        <v>HTTP Status: 201. Response trả về success = true cùng dữ liệu hợp lệ.</v>
+        <v>Ném ngoại lệ ApiError với status 4xx, mã lỗi 'ApiError'.</v>
       </c>
     </row>
     <row r="10" xml:space="preserve">
       <c r="A10" t="str">
-        <v>ACH-IT-03</v>
+        <v>ACH-AUTH-01</v>
       </c>
       <c r="B10" t="str">
-        <v>DELETE /api/admin/achievements/:id xóa danh hiệu thành công</v>
+        <v>Ghi nhận chính xác ID quản trị viên khi tạo danh hiệu mới</v>
       </c>
       <c r="C10" t="str">
-        <v>Kiểm thử chức năng chuẩn (Happy Path)</v>
+        <v>Kiểm thử phân quyền &amp; Bảo mật (Authorization &amp; Security 401/403)</v>
       </c>
       <c r="D10" t="str" xml:space="preserve">
-        <v xml:space="preserve">1. Thiết lập phiên đăng nhập / Mock quyền truy cập tương ứng.
-2. Gửi request HTTP DELETE tới endpoint /api/admin/achievements/:id.
-3. Xác thực mã trạng thái HTTP và cấu trúc JSON trả về.</v>
+        <v xml:space="preserve">1. Thiết lập Mock Repository / Database cho Service.
+2. Gọi method service.create() với tham số kiểm thử.
+3. Đối soát kết quả hoặc mã lỗi phát sinh.</v>
       </c>
       <c r="E10" t="str">
-        <v>Path param hoặc Payload chuẩn của achievement</v>
+        <v>Args: mockCreateAchievementInput, 99</v>
       </c>
       <c r="F10" t="str">
-        <v>HTTP Status: 200. Response trả về success = true cùng dữ liệu hợp lệ.</v>
+        <v>Hàm thực thi thành công, trả về đúng kiểu dữ liệu, các phương thức mock được gọi đúng tham số.</v>
       </c>
     </row>
     <row r="11" xml:space="preserve">
       <c r="A11" t="str">
-        <v>ACH-IT-04</v>
+        <v>ACH-AUTH-02</v>
       </c>
       <c r="B11" t="str">
-        <v>POST /api/admin/achievements thiếu title trả về 422</v>
+        <v>Ghi nhận chính xác ID quản trị viên khi cập nhật và xóa danh hiệu</v>
       </c>
       <c r="C11" t="str">
-        <v>Kiểm thử trường hợp biên &amp; Ngoại lệ (Negative / Bad Case)</v>
+        <v>Kiểm thử phân quyền &amp; Bảo mật (Authorization &amp; Security 401/403)</v>
       </c>
       <c r="D11" t="str" xml:space="preserve">
-        <v xml:space="preserve">1. Thiết lập phiên đăng nhập / Mock quyền truy cập tương ứng.
-2. Gửi request HTTP POST tới endpoint /api/admin/achievements.
-3. Xác thực mã trạng thái HTTP và cấu trúc JSON trả về.</v>
+        <v xml:space="preserve">1. Thiết lập Mock Repository / Database cho Service.
+2. Gọi method service.update() với tham số kiểm thử.
+3. Đối soát kết quả hoặc mã lỗi phát sinh.</v>
       </c>
       <c r="E11" t="str">
-        <v>{ requireXp: 100 }</v>
+        <v>Args: 1, { title: 'Super Title' }, 99</v>
       </c>
       <c r="F11" t="str">
-        <v>HTTP Status: 422. Báo lỗi validation hoặc bad request rõ ràng, không làm crash server.</v>
+        <v>Hàm thực thi thành công, trả về đúng kiểu dữ liệu, các phương thức mock được gọi đúng tham số.</v>
       </c>
     </row>
     <row r="12" xml:space="preserve">
       <c r="A12" t="str">
-        <v>ACH-IT-05</v>
+        <v>ACH-IT-AUTH-01</v>
       </c>
       <c r="B12" t="str">
-        <v>2 request xóa và tạo song song</v>
+        <v>GET /api/admin/achievements: Học viên (role: user) truy cập bị chặn với HTTP 403 Forbidden</v>
       </c>
       <c r="C12" t="str">
-        <v>Kiểm thử đụng độ đồng thời (Concurrency / Race Condition)</v>
+        <v>Kiểm thử phân quyền &amp; Bảo mật (Authorization &amp; Security 401/403)</v>
       </c>
       <c r="D12" t="str" xml:space="preserve">
         <v xml:space="preserve">1. Thiết lập phiên đăng nhập / Mock quyền truy cập tương ứng.
-2. Gửi request HTTP POST tới endpoint /api/admin/achievements.
+2. Gửi request HTTP GET tới endpoint /api/admin/achievements.
 3. Xác thực mã trạng thái HTTP và cấu trúc JSON trả về.</v>
       </c>
       <c r="E12" t="str">
-        <v>{ title: 'A3', requireXp: 50, requireStreak: 2 }</v>
+        <v>Path param hoặc Payload chuẩn của achievement</v>
       </c>
       <c r="F12" t="str">
-        <v>HTTP Status: 200. Response trả về success = true cùng dữ liệu hợp lệ.</v>
+        <v>HTTP Status: 403. Báo lỗi forbidden do tài khoản không có quyền truy cập thông tin quản trị.</v>
       </c>
     </row>
     <row r="13" xml:space="preserve">
       <c r="A13" t="str">
+        <v>ACH-IT-AUTH-02</v>
+      </c>
+      <c r="B13" t="str">
+        <v>POST /api/admin/achievements: Học viên (role: user) tạo danh hiệu bị chặn 403 Forbidden</v>
+      </c>
+      <c r="C13" t="str">
+        <v>Kiểm thử phân quyền &amp; Bảo mật (Authorization &amp; Security 401/403)</v>
+      </c>
+      <c r="D13" t="str" xml:space="preserve">
+        <v xml:space="preserve">1. Thiết lập phiên đăng nhập / Mock quyền truy cập tương ứng.
+2. Gửi request HTTP POST tới endpoint /api/admin/achievements:.
+3. Xác thực mã trạng thái HTTP và cấu trúc JSON trả về.</v>
+      </c>
+      <c r="E13" t="str">
+        <v>{ title: 'Hack Achievement', requireXp: 10, requireStreak: 1 }</v>
+      </c>
+      <c r="F13" t="str">
+        <v>HTTP Status: 403. Báo lỗi forbidden do tài khoản không có quyền truy cập thông tin quản trị.</v>
+      </c>
+    </row>
+    <row r="14" xml:space="preserve">
+      <c r="A14" t="str">
+        <v>ACH-IT-AUTH-03</v>
+      </c>
+      <c r="B14" t="str">
+        <v>PUT /api/admin/achievements/:id: Học viên (role: user) sửa danh hiệu bị chặn 403 Forbidden</v>
+      </c>
+      <c r="C14" t="str">
+        <v>Kiểm thử phân quyền &amp; Bảo mật (Authorization &amp; Security 401/403)</v>
+      </c>
+      <c r="D14" t="str" xml:space="preserve">
+        <v xml:space="preserve">1. Thiết lập phiên đăng nhập / Mock quyền truy cập tương ứng.
+2. Gửi request HTTP PUT tới endpoint /api/admin/achievements/:id:.
+3. Xác thực mã trạng thái HTTP và cấu trúc JSON trả về.</v>
+      </c>
+      <c r="E14" t="str">
+        <v>{ title: 'Hacked Title' }</v>
+      </c>
+      <c r="F14" t="str">
+        <v>HTTP Status: 403. Báo lỗi forbidden do tài khoản không có quyền truy cập thông tin quản trị.</v>
+      </c>
+    </row>
+    <row r="15" xml:space="preserve">
+      <c r="A15" t="str">
+        <v>ACH-IT-AUTH-04</v>
+      </c>
+      <c r="B15" t="str">
+        <v>DELETE /api/admin/achievements/:id: Học viên (role: user) xóa danh hiệu bị chặn 403 Forbidden</v>
+      </c>
+      <c r="C15" t="str">
+        <v>Kiểm thử phân quyền &amp; Bảo mật (Authorization &amp; Security 401/403)</v>
+      </c>
+      <c r="D15" t="str" xml:space="preserve">
+        <v xml:space="preserve">1. Thiết lập phiên đăng nhập / Mock quyền truy cập tương ứng.
+2. Gửi request HTTP DELETE tới endpoint /api/admin/achievements/1.
+3. Xác thực mã trạng thái HTTP và cấu trúc JSON trả về.</v>
+      </c>
+      <c r="E15" t="str">
+        <v>Path param hoặc Payload chuẩn của achievement</v>
+      </c>
+      <c r="F15" t="str">
+        <v>HTTP Status: 403. Báo lỗi forbidden do tài khoản không có quyền truy cập thông tin quản trị.</v>
+      </c>
+    </row>
+    <row r="16" xml:space="preserve">
+      <c r="A16" t="str">
+        <v>ACH-IT-AUTH-05</v>
+      </c>
+      <c r="B16" t="str">
+        <v>GET /api/admin/achievements: Request không gửi Token xác thực trả về 401 Unauthorized</v>
+      </c>
+      <c r="C16" t="str">
+        <v>Kiểm thử phân quyền &amp; Bảo mật (Authorization &amp; Security 401/403)</v>
+      </c>
+      <c r="D16" t="str" xml:space="preserve">
+        <v xml:space="preserve">1. Thiết lập phiên đăng nhập / Mock quyền truy cập tương ứng.
+2. Gửi request HTTP GET tới endpoint /api/admin/achievements.
+3. Xác thực mã trạng thái HTTP và cấu trúc JSON trả về.</v>
+      </c>
+      <c r="E16" t="str">
+        <v>Path param hoặc Payload chuẩn của achievement</v>
+      </c>
+      <c r="F16" t="str">
+        <v>HTTP Status: 401. Báo lỗi unauthorized do chưa cung cấp token xác thực.</v>
+      </c>
+    </row>
+    <row r="17" xml:space="preserve">
+      <c r="A17" t="str">
+        <v>ACH-IT-AUTH-06</v>
+      </c>
+      <c r="B17" t="str">
+        <v>DELETE /api/admin/achievements/:id: Request không gửi Token xác thực trả về 401 Unauthorized</v>
+      </c>
+      <c r="C17" t="str">
+        <v>Kiểm thử phân quyền &amp; Bảo mật (Authorization &amp; Security 401/403)</v>
+      </c>
+      <c r="D17" t="str" xml:space="preserve">
+        <v xml:space="preserve">1. Thiết lập phiên đăng nhập / Mock quyền truy cập tương ứng.
+2. Gửi request HTTP DELETE tới endpoint /api/admin/achievements/1.
+3. Xác thực mã trạng thái HTTP và cấu trúc JSON trả về.</v>
+      </c>
+      <c r="E17" t="str">
+        <v>Path param hoặc Payload chuẩn của achievement</v>
+      </c>
+      <c r="F17" t="str">
+        <v>HTTP Status: 401. Báo lỗi unauthorized do chưa cung cấp token xác thực.</v>
+      </c>
+    </row>
+    <row r="18" xml:space="preserve">
+      <c r="A18" t="str">
+        <v>ACH-IT-01</v>
+      </c>
+      <c r="B18" t="str">
+        <v>GET /api/admin/achievements trả về danh sách danh hiệu</v>
+      </c>
+      <c r="C18" t="str">
+        <v>Kiểm thử chức năng chuẩn (Happy Path)</v>
+      </c>
+      <c r="D18" t="str" xml:space="preserve">
+        <v xml:space="preserve">1. Thiết lập phiên đăng nhập / Mock quyền truy cập tương ứng.
+2. Gửi request HTTP GET tới endpoint /api/admin/achievements.
+3. Xác thực mã trạng thái HTTP và cấu trúc JSON trả về.</v>
+      </c>
+      <c r="E18" t="str">
+        <v>Path param hoặc Payload chuẩn của achievement</v>
+      </c>
+      <c r="F18" t="str">
+        <v>HTTP Status: 200. Response trả về success = true cùng dữ liệu hợp lệ.</v>
+      </c>
+    </row>
+    <row r="19" xml:space="preserve">
+      <c r="A19" t="str">
+        <v>ACH-IT-02</v>
+      </c>
+      <c r="B19" t="str">
+        <v>POST /api/admin/achievements tạo danh hiệu mới</v>
+      </c>
+      <c r="C19" t="str">
+        <v>Kiểm thử chức năng chuẩn (Happy Path)</v>
+      </c>
+      <c r="D19" t="str" xml:space="preserve">
+        <v xml:space="preserve">1. Thiết lập phiên đăng nhập / Mock quyền truy cập tương ứng.
+2. Gửi request HTTP POST tới endpoint /api/admin/achievements.
+3. Xác thực mã trạng thái HTTP và cấu trúc JSON trả về.</v>
+      </c>
+      <c r="E19" t="str">
+        <v>{ title: 'Bậc thầy', requireXp: 1000, requireStreak: 30 }</v>
+      </c>
+      <c r="F19" t="str">
+        <v>HTTP Status: 201. Response trả về success = true cùng dữ liệu hợp lệ.</v>
+      </c>
+    </row>
+    <row r="20" xml:space="preserve">
+      <c r="A20" t="str">
+        <v>ACH-IT-03</v>
+      </c>
+      <c r="B20" t="str">
+        <v>DELETE /api/admin/achievements/:id xóa danh hiệu thành công</v>
+      </c>
+      <c r="C20" t="str">
+        <v>Kiểm thử chức năng chuẩn (Happy Path)</v>
+      </c>
+      <c r="D20" t="str" xml:space="preserve">
+        <v xml:space="preserve">1. Thiết lập phiên đăng nhập / Mock quyền truy cập tương ứng.
+2. Gửi request HTTP DELETE tới endpoint /api/admin/achievements/1.
+3. Xác thực mã trạng thái HTTP và cấu trúc JSON trả về.</v>
+      </c>
+      <c r="E20" t="str">
+        <v>Path param hoặc Payload chuẩn của achievement</v>
+      </c>
+      <c r="F20" t="str">
+        <v>HTTP Status: 200. Response trả về success = true cùng dữ liệu hợp lệ.</v>
+      </c>
+    </row>
+    <row r="21" xml:space="preserve">
+      <c r="A21" t="str">
+        <v>ACH-IT-04</v>
+      </c>
+      <c r="B21" t="str">
+        <v>POST /api/admin/achievements thiếu title trả về 422</v>
+      </c>
+      <c r="C21" t="str">
+        <v>Kiểm thử trường hợp biên &amp; Ngoại lệ (Negative / Bad Case)</v>
+      </c>
+      <c r="D21" t="str" xml:space="preserve">
+        <v xml:space="preserve">1. Thiết lập phiên đăng nhập / Mock quyền truy cập tương ứng.
+2. Gửi request HTTP POST tới endpoint /api/admin/achievements.
+3. Xác thực mã trạng thái HTTP và cấu trúc JSON trả về.</v>
+      </c>
+      <c r="E21" t="str">
+        <v>{ requireXp: 100 }</v>
+      </c>
+      <c r="F21" t="str">
+        <v>HTTP Status: 422. Báo lỗi validation hoặc bad request rõ ràng, không làm crash server.</v>
+      </c>
+    </row>
+    <row r="22" xml:space="preserve">
+      <c r="A22" t="str">
+        <v>ACH-IT-05</v>
+      </c>
+      <c r="B22" t="str">
+        <v>PUT /api/admin/achievements/:id với id không phải số trả về 422</v>
+      </c>
+      <c r="C22" t="str">
+        <v>Kiểm thử trường hợp biên &amp; Ngoại lệ (Negative / Bad Case)</v>
+      </c>
+      <c r="D22" t="str" xml:space="preserve">
+        <v xml:space="preserve">1. Thiết lập phiên đăng nhập / Mock quyền truy cập tương ứng.
+2. Gửi request HTTP PUT tới endpoint /api/admin/achievements/:id.
+3. Xác thực mã trạng thái HTTP và cấu trúc JSON trả về.</v>
+      </c>
+      <c r="E22" t="str">
+        <v>{ title: 'Tên mới' }</v>
+      </c>
+      <c r="F22" t="str">
+        <v>HTTP Status: 422. Báo lỗi validation hoặc bad request rõ ràng, không làm crash server.</v>
+      </c>
+    </row>
+    <row r="23" xml:space="preserve">
+      <c r="A23" t="str">
+        <v>ACH-IT-RACE-01</v>
+      </c>
+      <c r="B23" t="str">
+        <v>Đụng độ Cập nhật &amp; Xóa đồng thời: 1 request thành công, 1 request gặp danh hiệu đã xóa trả về 404</v>
+      </c>
+      <c r="C23" t="str">
+        <v>Kiểm thử đụng độ đồng thời (Concurrency / Race Condition - Update vs Delete)</v>
+      </c>
+      <c r="D23" t="str" xml:space="preserve">
+        <v xml:space="preserve">1. Thiết lập phiên đăng nhập / Mock quyền truy cập tương ứng.
+2. Gửi request HTTP DELETE tới endpoint /api/admin/achievements/10.
+3. Xác thực mã trạng thái HTTP và cấu trúc JSON trả về.</v>
+      </c>
+      <c r="E23" t="str">
+        <v>{ title: 'Updated' }</v>
+      </c>
+      <c r="F23" t="str">
+        <v>HTTP Status: 200. Response trả về success = true cùng dữ liệu hợp lệ.</v>
+      </c>
+    </row>
+    <row r="24" xml:space="preserve">
+      <c r="A24" t="str">
+        <v>ACH-IT-RACE-02</v>
+      </c>
+      <c r="B24" t="str">
+        <v>Đụng độ Update tới trước - Delete xen ngang: Cập nhật không làm vô hiệu hóa kết quả xóa</v>
+      </c>
+      <c r="C24" t="str">
+        <v>Kiểm thử đụng độ đồng thời (Concurrency / Race Condition - Update vs Delete)</v>
+      </c>
+      <c r="D24" t="str" xml:space="preserve">
+        <v xml:space="preserve">1. Thiết lập phiên đăng nhập / Mock quyền truy cập tương ứng.
+2. Gửi request HTTP DELETE tới endpoint xen.
+3. Xác thực mã trạng thái HTTP và cấu trúc JSON trả về.</v>
+      </c>
+      <c r="E24" t="str">
+        <v>{ title: 'Title Cập Nhật' }</v>
+      </c>
+      <c r="F24" t="str">
+        <v>HTTP Status: 404. Báo lỗi student_not_found do bản ghi đã bị xóa hoặc không tồn tại.</v>
+      </c>
+    </row>
+    <row r="25" xml:space="preserve">
+      <c r="A25" t="str">
+        <v>ACH-IT-RACE-03</v>
+      </c>
+      <c r="B25" t="str">
+        <v>Hai Admin cùng gửi request cập nhật cùng một danh hiệu đồng thời</v>
+      </c>
+      <c r="C25" t="str">
+        <v>Kiểm thử đụng độ đồng thời (Concurrency / Race Condition - Update vs Delete)</v>
+      </c>
+      <c r="D25" t="str" xml:space="preserve">
+        <v xml:space="preserve">1. Thiết lập phiên đăng nhập / Mock quyền truy cập tương ứng.
+2. Gửi request HTTP PUT tới endpoint /api/admin/achievements/1.
+3. Xác thực mã trạng thái HTTP và cấu trúc JSON trả về.</v>
+      </c>
+      <c r="E25" t="str">
+        <v>{ title: 'Admin 1 update' }</v>
+      </c>
+      <c r="F25" t="str">
+        <v>HTTP Status: 200. Response trả về success = true cùng dữ liệu hợp lệ.</v>
+      </c>
+    </row>
+    <row r="26" xml:space="preserve">
+      <c r="A26" t="str">
         <v>ACH-IT-06</v>
       </c>
-      <c r="B13" t="str">
+      <c r="B26" t="str">
         <v>Mất kết nối DB khi lấy danh sách trả về 500</v>
       </c>
-      <c r="C13" t="str">
-        <v>Kiểm thử mất kết nối mạng &amp; Lỗi hệ thống (Network &amp; System Error)</v>
-      </c>
-      <c r="D13" t="str" xml:space="preserve">
+      <c r="C26" t="str">
+        <v>Kiểm thử toàn vẹn dữ liệu &amp; Xung đột (Data Conflict / Rollback)</v>
+      </c>
+      <c r="D26" t="str" xml:space="preserve">
         <v xml:space="preserve">1. Thiết lập phiên đăng nhập / Mock quyền truy cập tương ứng.
 2. Gửi request HTTP GET tới endpoint /api/admin/achievements.
 3. Xác thực mã trạng thái HTTP và cấu trúc JSON trả về.</v>
       </c>
-      <c r="E13" t="str">
+      <c r="E26" t="str">
         <v>Path param hoặc Payload chuẩn của achievement</v>
       </c>
-      <c r="F13" t="str">
+      <c r="F26" t="str">
         <v>HTTP Status: 500. Hệ thống bắt lỗi thông qua error-handler, trả về HTTP 500 an toàn.</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:F13"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:F26"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F9"/>
+  <dimension ref="A1:F15"/>
   <cols>
-    <col min="1" max="1" width="15.83203125" customWidth="1"/>
-    <col min="2" max="2" width="45.83203125" customWidth="1"/>
-    <col min="3" max="3" width="35.83203125" customWidth="1"/>
+    <col min="1" max="1" width="18.83203125" customWidth="1"/>
+    <col min="2" max="2" width="48.83203125" customWidth="1"/>
+    <col min="3" max="3" width="40.83203125" customWidth="1"/>
     <col min="4" max="4" width="45.83203125" customWidth="1"/>
     <col min="5" max="5" width="35.83203125" customWidth="1"/>
-    <col min="6" max="6" width="45.83203125" customWidth="1"/>
+    <col min="6" max="6" width="48.83203125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -5959,12 +6707,12 @@
         <v>Kiểm thử chức năng chuẩn (Happy Path)</v>
       </c>
       <c r="D2" t="str" xml:space="preserve">
-        <v xml:space="preserve">1. Khởi tạo Service với Mock Repository / Prisma Client.
-2. Kích hoạt hàm nghiệp vụ tương ứng của activity-log.
-3. Kiểm tra giá trị trả về hoặc bắt exception.</v>
+        <v xml:space="preserve">1. Thiết lập Mock Repository / Database cho Service.
+2. Gọi method service.getActivities() với tham số kiểm thử.
+3. Đối soát kết quả hoặc mã lỗi phát sinh.</v>
       </c>
       <c r="E2" t="str">
-        <v>Dữ liệu test fixture trong activity-log.mock.ts</v>
+        <v>Args: 1, 20</v>
       </c>
       <c r="F2" t="str">
         <v>Hàm thực thi thành công, trả về đúng kiểu dữ liệu, các phương thức mock được gọi đúng tham số.</v>
@@ -5981,12 +6729,12 @@
         <v>Kiểm thử chức năng chuẩn (Happy Path)</v>
       </c>
       <c r="D3" t="str" xml:space="preserve">
-        <v xml:space="preserve">1. Khởi tạo Service với Mock Repository / Prisma Client.
-2. Kích hoạt hàm nghiệp vụ tương ứng của activity-log.
-3. Kiểm tra giá trị trả về hoặc bắt exception.</v>
+        <v xml:space="preserve">1. Thiết lập Mock Repository / Database cho Service.
+2. Gọi method service.getLoginLogs() với tham số kiểm thử.
+3. Đối soát kết quả hoặc mã lỗi phát sinh.</v>
       </c>
       <c r="E3" t="str">
-        <v>Dữ liệu test fixture trong activity-log.mock.ts</v>
+        <v>Args: 1, 20</v>
       </c>
       <c r="F3" t="str">
         <v>Hàm thực thi thành công, trả về đúng kiểu dữ liệu, các phương thức mock được gọi đúng tham số.</v>
@@ -6003,12 +6751,12 @@
         <v>Kiểm thử trường hợp biên &amp; Ngoại lệ (Negative / Bad Case)</v>
       </c>
       <c r="D4" t="str" xml:space="preserve">
-        <v xml:space="preserve">1. Khởi tạo Service với Mock Repository / Prisma Client.
-2. Kích hoạt hàm nghiệp vụ tương ứng của activity-log.
-3. Kiểm tra giá trị trả về hoặc bắt exception.</v>
+        <v xml:space="preserve">1. Thiết lập Mock Repository / Database cho Service.
+2. Gọi method service.getActivities() với tham số kiểm thử.
+3. Đối soát kết quả hoặc mã lỗi phát sinh.</v>
       </c>
       <c r="E4" t="str">
-        <v>Dữ liệu test fixture trong activity-log.mock.ts</v>
+        <v>Args: 1, 20, 'unknown_keyword'</v>
       </c>
       <c r="F4" t="str">
         <v>Ném ngoại lệ ApiError với status 4xx, mã lỗi 'ApiError'.</v>
@@ -6016,13 +6764,13 @@
     </row>
     <row r="5" xml:space="preserve">
       <c r="A5" t="str">
-        <v>LOG-03</v>
+        <v>LOG-AUTH-01</v>
       </c>
       <c r="B5" t="str">
-        <v>Nhiều Admin cùng truy vấn logs đồng thời</v>
+        <v>Bảo mật dữ liệu: Lọc nhật ký hoạt động theo actionType và phân quyền quản trị viên</v>
       </c>
       <c r="C5" t="str">
-        <v>Kiểm thử đụng độ đồng thời (Concurrency / Race Condition)</v>
+        <v>Kiểm thử phân quyền &amp; Bảo mật (Authorization &amp; Security 401/403)</v>
       </c>
       <c r="D5" t="str" xml:space="preserve">
         <v xml:space="preserve">1. Thiết lập Mock Repository / Database cho Service.
@@ -6030,7 +6778,7 @@
 3. Đối soát kết quả hoặc mã lỗi phát sinh.</v>
       </c>
       <c r="E5" t="str">
-        <v>Args: 1, 10</v>
+        <v>Args: 1, 20, undefined, 'ADMIN_UPDATE'</v>
       </c>
       <c r="F5" t="str">
         <v>Hàm thực thi thành công, trả về đúng kiểu dữ liệu, các phương thức mock được gọi đúng tham số.</v>
@@ -6038,79 +6786,79 @@
     </row>
     <row r="6" xml:space="preserve">
       <c r="A6" t="str">
-        <v>LOG-05</v>
+        <v>LOG-AUTH-02</v>
       </c>
       <c r="B6" t="str">
-        <v>Mất kết nối DB khi truy vấn logs ném lỗi hệ thống</v>
+        <v>Bảo mật dữ liệu: Nhật ký đăng nhập ghi nhận đầy đủ địa chỉ IP và thông tin xác thực</v>
       </c>
       <c r="C6" t="str">
-        <v>Kiểm thử mất kết nối mạng &amp; Lỗi hệ thống (Network &amp; System Error)</v>
+        <v>Kiểm thử phân quyền &amp; Bảo mật (Authorization &amp; Security 401/403)</v>
       </c>
       <c r="D6" t="str" xml:space="preserve">
         <v xml:space="preserve">1. Thiết lập Mock Repository / Database cho Service.
-2. Gọi method service.getActivities() với tham số kiểm thử.
+2. Gọi method service.getLoginLogs() với tham số kiểm thử.
 3. Đối soát kết quả hoặc mã lỗi phát sinh.</v>
       </c>
       <c r="E6" t="str">
-        <v>Args: 1, 20</v>
+        <v>Args: 1, 20, '127.0.0.1'</v>
       </c>
       <c r="F6" t="str">
-        <v>Ném ngoại lệ ApiError với status 4xx, mã lỗi 'ApiError'.</v>
+        <v>Hàm thực thi thành công, trả về đúng kiểu dữ liệu, các phương thức mock được gọi đúng tham số.</v>
       </c>
     </row>
     <row r="7" xml:space="preserve">
       <c r="A7" t="str">
-        <v>LOG-IT-01</v>
+        <v>LOG-05</v>
       </c>
       <c r="B7" t="str">
-        <v>GET /api/admin/logs/activities trả về danh sách lịch sử hoạt động</v>
+        <v>Mất kết nối DB khi truy vấn logs ném lỗi hệ thống</v>
       </c>
       <c r="C7" t="str">
-        <v>Kiểm thử chức năng chuẩn (Happy Path)</v>
+        <v>Kiểm thử toàn vẹn dữ liệu &amp; Xung đột (Data Conflict / Rollback)</v>
       </c>
       <c r="D7" t="str" xml:space="preserve">
-        <v xml:space="preserve">1. Thiết lập phiên đăng nhập / Mock quyền truy cập tương ứng.
-2. Gửi request HTTP GET tới endpoint /api/admin/logs/activities.
-3. Xác thực mã trạng thái HTTP và cấu trúc JSON trả về.</v>
+        <v xml:space="preserve">1. Thiết lập Mock Repository / Database cho Service.
+2. Gọi method service.getActivities() với tham số kiểm thử.
+3. Đối soát kết quả hoặc mã lỗi phát sinh.</v>
       </c>
       <c r="E7" t="str">
-        <v>Path param hoặc Payload chuẩn của activity-log</v>
+        <v>Args: 1, 20</v>
       </c>
       <c r="F7" t="str">
-        <v>HTTP Status: 200. Response trả về success = true cùng dữ liệu hợp lệ.</v>
+        <v>Ném ngoại lệ ApiError với status 4xx, mã lỗi 'ApiError'.</v>
       </c>
     </row>
     <row r="8" xml:space="preserve">
       <c r="A8" t="str">
-        <v>LOG-IT-02</v>
+        <v>LOG-IT-AUTH-01</v>
       </c>
       <c r="B8" t="str">
-        <v>GET /api/admin/logs/login-logs trả về danh sách lịch sử đăng nhập</v>
+        <v>GET /api/admin/logs/activities: Học viên (role: user) truy cập bị chặn với HTTP 403 Forbidden</v>
       </c>
       <c r="C8" t="str">
-        <v>Kiểm thử chức năng chuẩn (Happy Path)</v>
+        <v>Kiểm thử phân quyền &amp; Bảo mật (Authorization &amp; Security 401/403)</v>
       </c>
       <c r="D8" t="str" xml:space="preserve">
         <v xml:space="preserve">1. Thiết lập phiên đăng nhập / Mock quyền truy cập tương ứng.
-2. Gửi request HTTP GET tới endpoint /api/admin/logs/login-logs.
+2. Gửi request HTTP GET tới endpoint /api/admin/logs/activities.
 3. Xác thực mã trạng thái HTTP và cấu trúc JSON trả về.</v>
       </c>
       <c r="E8" t="str">
         <v>Path param hoặc Payload chuẩn của activity-log</v>
       </c>
       <c r="F8" t="str">
-        <v>HTTP Status: 200. Response trả về success = true cùng dữ liệu hợp lệ.</v>
+        <v>HTTP Status: 403. Báo lỗi forbidden do tài khoản không có quyền truy cập thông tin quản trị.</v>
       </c>
     </row>
     <row r="9" xml:space="preserve">
       <c r="A9" t="str">
-        <v>LOG-IT-03</v>
+        <v>LOG-IT-AUTH-02</v>
       </c>
       <c r="B9" t="str">
-        <v>Mất kết nối DB khi truy vấn login logs trả về 500</v>
+        <v>GET /api/admin/logs/login-logs: Học viên (role: user) truy cập bị chặn với HTTP 403 Forbidden</v>
       </c>
       <c r="C9" t="str">
-        <v>Kiểm thử mất kết nối mạng &amp; Lỗi hệ thống (Network &amp; System Error)</v>
+        <v>Kiểm thử phân quyền &amp; Bảo mật (Authorization &amp; Security 401/403)</v>
       </c>
       <c r="D9" t="str" xml:space="preserve">
         <v xml:space="preserve">1. Thiết lập phiên đăng nhập / Mock quyền truy cập tương ứng.
@@ -6121,26 +6869,158 @@
         <v>Path param hoặc Payload chuẩn của activity-log</v>
       </c>
       <c r="F9" t="str">
+        <v>HTTP Status: 403. Báo lỗi forbidden do tài khoản không có quyền truy cập thông tin quản trị.</v>
+      </c>
+    </row>
+    <row r="10" xml:space="preserve">
+      <c r="A10" t="str">
+        <v>LOG-IT-AUTH-03</v>
+      </c>
+      <c r="B10" t="str">
+        <v>GET /api/admin/logs/activities: Request không gửi Token xác thực trả về 401 Unauthorized</v>
+      </c>
+      <c r="C10" t="str">
+        <v>Kiểm thử phân quyền &amp; Bảo mật (Authorization &amp; Security 401/403)</v>
+      </c>
+      <c r="D10" t="str" xml:space="preserve">
+        <v xml:space="preserve">1. Thiết lập phiên đăng nhập / Mock quyền truy cập tương ứng.
+2. Gửi request HTTP GET tới endpoint /api/admin/logs/activities.
+3. Xác thực mã trạng thái HTTP và cấu trúc JSON trả về.</v>
+      </c>
+      <c r="E10" t="str">
+        <v>Path param hoặc Payload chuẩn của activity-log</v>
+      </c>
+      <c r="F10" t="str">
+        <v>HTTP Status: 401. Báo lỗi unauthorized do chưa cung cấp token xác thực.</v>
+      </c>
+    </row>
+    <row r="11" xml:space="preserve">
+      <c r="A11" t="str">
+        <v>LOG-IT-AUTH-04</v>
+      </c>
+      <c r="B11" t="str">
+        <v>GET /api/admin/logs/login-logs: Request không gửi Token xác thực trả về 401 Unauthorized</v>
+      </c>
+      <c r="C11" t="str">
+        <v>Kiểm thử phân quyền &amp; Bảo mật (Authorization &amp; Security 401/403)</v>
+      </c>
+      <c r="D11" t="str" xml:space="preserve">
+        <v xml:space="preserve">1. Thiết lập phiên đăng nhập / Mock quyền truy cập tương ứng.
+2. Gửi request HTTP GET tới endpoint /api/admin/logs/login-logs.
+3. Xác thực mã trạng thái HTTP và cấu trúc JSON trả về.</v>
+      </c>
+      <c r="E11" t="str">
+        <v>Path param hoặc Payload chuẩn của activity-log</v>
+      </c>
+      <c r="F11" t="str">
+        <v>HTTP Status: 401. Báo lỗi unauthorized do chưa cung cấp token xác thực.</v>
+      </c>
+    </row>
+    <row r="12" xml:space="preserve">
+      <c r="A12" t="str">
+        <v>LOG-IT-01</v>
+      </c>
+      <c r="B12" t="str">
+        <v>GET /api/admin/logs/activities trả về danh sách lịch sử hoạt động</v>
+      </c>
+      <c r="C12" t="str">
+        <v>Kiểm thử chức năng chuẩn (Happy Path)</v>
+      </c>
+      <c r="D12" t="str" xml:space="preserve">
+        <v xml:space="preserve">1. Thiết lập phiên đăng nhập / Mock quyền truy cập tương ứng.
+2. Gửi request HTTP GET tới endpoint /api/admin/logs/activities?page=1&amp;limit=20.
+3. Xác thực mã trạng thái HTTP và cấu trúc JSON trả về.</v>
+      </c>
+      <c r="E12" t="str">
+        <v>Query parameters: page=1&amp;limit=20</v>
+      </c>
+      <c r="F12" t="str">
+        <v>HTTP Status: 200. Response trả về success = true cùng dữ liệu hợp lệ.</v>
+      </c>
+    </row>
+    <row r="13" xml:space="preserve">
+      <c r="A13" t="str">
+        <v>LOG-IT-02</v>
+      </c>
+      <c r="B13" t="str">
+        <v>GET /api/admin/logs/login-logs trả về danh sách lịch sử đăng nhập</v>
+      </c>
+      <c r="C13" t="str">
+        <v>Kiểm thử chức năng chuẩn (Happy Path)</v>
+      </c>
+      <c r="D13" t="str" xml:space="preserve">
+        <v xml:space="preserve">1. Thiết lập phiên đăng nhập / Mock quyền truy cập tương ứng.
+2. Gửi request HTTP GET tới endpoint /api/admin/logs/login-logs.
+3. Xác thực mã trạng thái HTTP và cấu trúc JSON trả về.</v>
+      </c>
+      <c r="E13" t="str">
+        <v>Path param hoặc Payload chuẩn của activity-log</v>
+      </c>
+      <c r="F13" t="str">
+        <v>HTTP Status: 200. Response trả về success = true cùng dữ liệu hợp lệ.</v>
+      </c>
+    </row>
+    <row r="14" xml:space="preserve">
+      <c r="A14" t="str">
+        <v>LOG-IT-03</v>
+      </c>
+      <c r="B14" t="str">
+        <v>GET /api/admin/logs/activities với page âm hoặc không hợp lệ trả về kết quả an toàn</v>
+      </c>
+      <c r="C14" t="str">
+        <v>Kiểm thử trường hợp biên &amp; Ngoại lệ (Negative / Bad Case)</v>
+      </c>
+      <c r="D14" t="str" xml:space="preserve">
+        <v xml:space="preserve">1. Thiết lập phiên đăng nhập / Mock quyền truy cập tương ứng.
+2. Gửi request HTTP GET tới endpoint /api/admin/logs/activities?page=-1.
+3. Xác thực mã trạng thái HTTP và cấu trúc JSON trả về.</v>
+      </c>
+      <c r="E14" t="str">
+        <v>Query parameters: page=-1</v>
+      </c>
+      <c r="F14" t="str">
+        <v>HTTP Status: 200. Response trả về success = true cùng dữ liệu hợp lệ.</v>
+      </c>
+    </row>
+    <row r="15" xml:space="preserve">
+      <c r="A15" t="str">
+        <v>LOG-IT-04</v>
+      </c>
+      <c r="B15" t="str">
+        <v>Mất kết nối DB khi truy vấn login logs trả về 500</v>
+      </c>
+      <c r="C15" t="str">
+        <v>Kiểm thử mất kết nối mạng &amp; Lỗi hệ thống (Network &amp; System Error)</v>
+      </c>
+      <c r="D15" t="str" xml:space="preserve">
+        <v xml:space="preserve">1. Thiết lập phiên đăng nhập / Mock quyền truy cập tương ứng.
+2. Gửi request HTTP GET tới endpoint /api/admin/logs/login-logs.
+3. Xác thực mã trạng thái HTTP và cấu trúc JSON trả về.</v>
+      </c>
+      <c r="E15" t="str">
+        <v>Path param hoặc Payload chuẩn của activity-log</v>
+      </c>
+      <c r="F15" t="str">
         <v>HTTP Status: 500. Hệ thống bắt lỗi thông qua error-handler, trả về HTTP 500 an toàn.</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:F9"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:F15"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F20"/>
+  <dimension ref="A1:F30"/>
   <cols>
-    <col min="1" max="1" width="15.83203125" customWidth="1"/>
-    <col min="2" max="2" width="45.83203125" customWidth="1"/>
-    <col min="3" max="3" width="35.83203125" customWidth="1"/>
+    <col min="1" max="1" width="18.83203125" customWidth="1"/>
+    <col min="2" max="2" width="48.83203125" customWidth="1"/>
+    <col min="3" max="3" width="40.83203125" customWidth="1"/>
     <col min="4" max="4" width="45.83203125" customWidth="1"/>
     <col min="5" max="5" width="35.83203125" customWidth="1"/>
-    <col min="6" max="6" width="45.83203125" customWidth="1"/>
+    <col min="6" max="6" width="48.83203125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -6314,7 +7194,7 @@
         <v>Dữ liệu test fixture trong auth.mock.ts</v>
       </c>
       <c r="F8" t="str">
-        <v>Ném ngoại lệ ApiError với status 4xx, mã lỗi 'ApiError'.</v>
+        <v>Ném ngoại lệ ApiError với status 403, mã lỗi 'ApiError'.</v>
       </c>
     </row>
     <row r="9" xml:space="preserve">
@@ -6325,7 +7205,7 @@
         <v>Phát hiện đụng độ / replay refresh token: &gt;= 3 lần refresh/phút hủy toàn bộ phiên</v>
       </c>
       <c r="C9" t="str">
-        <v>Kiểm thử đụng độ đồng thời (Concurrency / Race Condition)</v>
+        <v>Kiểm thử đụng độ đồng thời (Concurrency / Race Condition - Update vs Delete)</v>
       </c>
       <c r="D9" t="str" xml:space="preserve">
         <v xml:space="preserve">1. Khởi tạo Service với Mock Repository / Prisma Client.
@@ -6336,7 +7216,7 @@
         <v>Dữ liệu test fixture trong auth.mock.ts</v>
       </c>
       <c r="F9" t="str">
-        <v>Hàm thực thi thành công, trả về đúng kiểu dữ liệu, các phương thức mock được gọi đúng tham số.</v>
+        <v>Ném ngoại lệ ApiError với status 429, mã lỗi 'ApiError'.</v>
       </c>
     </row>
     <row r="10" xml:space="preserve">
@@ -6347,7 +7227,7 @@
         <v>Xung đột dữ liệu: Chặn đăng ký khi trùng Email đã tồn tại</v>
       </c>
       <c r="C10" t="str">
-        <v>Kiểm thử toàn vẹn dữ liệu &amp; Xung đột (Data Conflict / Rollback)</v>
+        <v>Kiểm thử phân quyền &amp; Bảo mật (Authorization &amp; Security 401/403)</v>
       </c>
       <c r="D10" t="str" xml:space="preserve">
         <v xml:space="preserve">1. Khởi tạo Service với Mock Repository / Prisma Client.
@@ -6369,7 +7249,7 @@
         <v>Xung đột dữ liệu: Chặn đăng ký khi trùng Tên đăng nhập</v>
       </c>
       <c r="C11" t="str">
-        <v>Kiểm thử toàn vẹn dữ liệu &amp; Xung đột (Data Conflict / Rollback)</v>
+        <v>Kiểm thử phân quyền &amp; Bảo mật (Authorization &amp; Security 401/403)</v>
       </c>
       <c r="D11" t="str" xml:space="preserve">
         <v xml:space="preserve">1. Khởi tạo Service với Mock Repository / Prisma Client.
@@ -6402,7 +7282,7 @@
         <v>Dữ liệu test fixture trong auth.mock.ts</v>
       </c>
       <c r="F12" t="str">
-        <v>Hàm thực thi thành công, trả về đúng kiểu dữ liệu, các phương thức mock được gọi đúng tham số.</v>
+        <v>Ném ngoại lệ ApiError với status 401, mã lỗi 'token_revoked'.</v>
       </c>
     </row>
     <row r="13" xml:space="preserve">
@@ -6429,123 +7309,123 @@
     </row>
     <row r="14" xml:space="preserve">
       <c r="A14" t="str">
-        <v>AUTH-IT-01</v>
+        <v>AUTH-SEC-01</v>
       </c>
       <c r="B14" t="str">
-        <v>POST /api/auth/register thành công với mã 201</v>
+        <v>Thu hồi Session an toàn: Logout đưa Access Token vào danh sách đen (revoked_token) và đánh dấu Refresh Token isRevoked = true</v>
       </c>
       <c r="C14" t="str">
         <v>Kiểm thử chức năng chuẩn (Happy Path)</v>
       </c>
       <c r="D14" t="str" xml:space="preserve">
-        <v xml:space="preserve">1. Thiết lập phiên đăng nhập / Mock quyền truy cập tương ứng.
-2. Gửi request HTTP POST tới endpoint /api/auth/register.
-3. Xác thực mã trạng thái HTTP và cấu trúc JSON trả về.</v>
+        <v xml:space="preserve">1. Khởi tạo Service với Mock Repository / Prisma Client.
+2. Kích hoạt hàm nghiệp vụ tương ứng của auth.
+3. Kiểm tra giá trị trả về hoặc bắt exception.</v>
       </c>
       <c r="E14" t="str">
-        <v>Path param hoặc Payload chuẩn của auth</v>
+        <v>Dữ liệu test fixture trong auth.mock.ts</v>
       </c>
       <c r="F14" t="str">
-        <v>HTTP Status: 200. Response trả về success = true cùng dữ liệu hợp lệ.</v>
+        <v>Hàm thực thi thành công, trả về đúng kiểu dữ liệu, các phương thức mock được gọi đúng tham số.</v>
       </c>
     </row>
     <row r="15" xml:space="preserve">
       <c r="A15" t="str">
-        <v>AUTH-IT-02</v>
+        <v>AUTH-SEC-02</v>
       </c>
       <c r="B15" t="str">
-        <v>POST /api/auth/login thành công với mã 200</v>
+        <v>Chống Replay Refresh Token: Kẻ tấn công dùng Refresh Token đã bị revoke để lấy token mới -&gt; Bị từ chối 401 và toàn bộ Session bị triệt hạ</v>
       </c>
       <c r="C15" t="str">
-        <v>Kiểm thử chức năng chuẩn (Happy Path)</v>
+        <v>Kiểm thử phân quyền &amp; Bảo mật (Authorization &amp; Security 401/403)</v>
       </c>
       <c r="D15" t="str" xml:space="preserve">
-        <v xml:space="preserve">1. Thiết lập phiên đăng nhập / Mock quyền truy cập tương ứng.
-2. Gửi request HTTP POST tới endpoint /api/auth/login.
-3. Xác thực mã trạng thái HTTP và cấu trúc JSON trả về.</v>
+        <v xml:space="preserve">1. Khởi tạo Service với Mock Repository / Prisma Client.
+2. Kích hoạt hàm nghiệp vụ tương ứng của auth.
+3. Kiểm tra giá trị trả về hoặc bắt exception.</v>
       </c>
       <c r="E15" t="str">
-        <v>Path param hoặc Payload chuẩn của auth</v>
+        <v>Dữ liệu test fixture trong auth.mock.ts</v>
       </c>
       <c r="F15" t="str">
-        <v>HTTP Status: 200. Response trả về success = true cùng dữ liệu hợp lệ.</v>
+        <v>Ném ngoại lệ ApiError với status 401, mã lỗi 'token_revoked'.</v>
       </c>
     </row>
     <row r="16" xml:space="preserve">
       <c r="A16" t="str">
-        <v>AUTH-IT-03</v>
+        <v>AUTH-SEC-03</v>
       </c>
       <c r="B16" t="str">
-        <v>POST /api/auth/login thiếu mật khẩu trả về 422 Validation Error</v>
+        <v>Chống dùng lại Access Token cũ sau khi Refresh (Token Rotation): Access Token cũ trước đó bị đưa vào blacklist ngay lập tức</v>
       </c>
       <c r="C16" t="str">
-        <v>Kiểm thử trường hợp biên &amp; Ngoại lệ (Negative / Bad Case)</v>
+        <v>Kiểm thử chức năng chuẩn (Happy Path)</v>
       </c>
       <c r="D16" t="str" xml:space="preserve">
-        <v xml:space="preserve">1. Thiết lập phiên đăng nhập / Mock quyền truy cập tương ứng.
-2. Gửi request HTTP POST tới endpoint /api/auth/login.
-3. Xác thực mã trạng thái HTTP và cấu trúc JSON trả về.</v>
+        <v xml:space="preserve">1. Khởi tạo Service với Mock Repository / Prisma Client.
+2. Kích hoạt hàm nghiệp vụ tương ứng của auth.
+3. Kiểm tra giá trị trả về hoặc bắt exception.</v>
       </c>
       <c r="E16" t="str">
-        <v>{ identifier: 'valid@example.com', // thiếu password }</v>
+        <v>Dữ liệu test fixture trong auth.mock.ts</v>
       </c>
       <c r="F16" t="str">
-        <v xml:space="preserve">HTTP Status: 400 / 422. </v>
+        <v>Hàm thực thi thành công, trả về đúng kiểu dữ liệu, các phương thức mock được gọi đúng tham số.</v>
       </c>
     </row>
     <row r="17" xml:space="preserve">
       <c r="A17" t="str">
-        <v>AUTH-IT-04</v>
+        <v>AUTH-SEC-04</v>
       </c>
       <c r="B17" t="str">
-        <v>POST /api/auth/register email không đúng định dạng trả về 422</v>
+        <v>Phát hiện tấn công Brute-force/Spam Refresh: Hủy tức thì toàn bộ Session và đưa cả Access Token lẫn Refresh Token vào blacklist khi tần suất &gt;= 3 lần/phút</v>
       </c>
       <c r="C17" t="str">
-        <v>Kiểm thử trường hợp biên &amp; Ngoại lệ (Negative / Bad Case)</v>
+        <v>Kiểm thử đụng độ đồng thời (Concurrency / Race Condition - Update vs Delete)</v>
       </c>
       <c r="D17" t="str" xml:space="preserve">
-        <v xml:space="preserve">1. Thiết lập phiên đăng nhập / Mock quyền truy cập tương ứng.
-2. Gửi request HTTP POST tới endpoint /api/auth/register.
-3. Xác thực mã trạng thái HTTP và cấu trúc JSON trả về.</v>
+        <v xml:space="preserve">1. Khởi tạo Service với Mock Repository / Prisma Client.
+2. Kích hoạt hàm nghiệp vụ tương ứng của auth.
+3. Kiểm tra giá trị trả về hoặc bắt exception.</v>
       </c>
       <c r="E17" t="str">
-        <v>{ username: 'invalidmail', email: 'not-an-email', password: 'Password123@', }</v>
+        <v>Dữ liệu test fixture trong auth.mock.ts</v>
       </c>
       <c r="F17" t="str">
-        <v xml:space="preserve">HTTP Status: 400 / 422. </v>
+        <v>Ném ngoại lệ ApiError với status 429, mã lỗi 'too_many_refresh_requests'.</v>
       </c>
     </row>
     <row r="18" xml:space="preserve">
       <c r="A18" t="str">
-        <v>AUTH-IT-05</v>
+        <v>AUTH-SEC-05</v>
       </c>
       <c r="B18" t="str">
-        <v>POST /api/auth/refresh khi session bị spam &gt; 3 lần/phút trả về 429</v>
+        <v>Ngăn chặn phiên làm việc của tài khoản bị khóa: Refresh token của user có isLocked = true bị từ chối 403 account_locked</v>
       </c>
       <c r="C18" t="str">
-        <v>Kiểm thử đụng độ đồng thời (Concurrency / Race Condition)</v>
+        <v>Kiểm thử phân quyền &amp; Bảo mật (Authorization &amp; Security 401/403)</v>
       </c>
       <c r="D18" t="str" xml:space="preserve">
-        <v xml:space="preserve">1. Thiết lập phiên đăng nhập / Mock quyền truy cập tương ứng.
-2. Gửi request HTTP POST tới endpoint /api/auth/refresh.
-3. Xác thực mã trạng thái HTTP và cấu trúc JSON trả về.</v>
+        <v xml:space="preserve">1. Khởi tạo Service với Mock Repository / Prisma Client.
+2. Kích hoạt hàm nghiệp vụ tương ứng của auth.
+3. Kiểm tra giá trị trả về hoặc bắt exception.</v>
       </c>
       <c r="E18" t="str">
-        <v>{ refreshToken: 'spam_refresh_token' }</v>
+        <v>Dữ liệu test fixture trong auth.mock.ts</v>
       </c>
       <c r="F18" t="str">
-        <v xml:space="preserve">HTTP Status: 429. </v>
+        <v>Ném ngoại lệ ApiError với status 403, mã lỗi 'account_locked'.</v>
       </c>
     </row>
     <row r="19" xml:space="preserve">
       <c r="A19" t="str">
-        <v>AUTH-IT-06</v>
+        <v>AUTH-IT-01</v>
       </c>
       <c r="B19" t="str">
-        <v>POST /api/auth/register khi email đã tồn tại trả về 409 Conflict</v>
+        <v>POST /api/auth/register thành công với mã 201</v>
       </c>
       <c r="C19" t="str">
-        <v>Kiểm thử toàn vẹn dữ liệu &amp; Xung đột (Data Conflict / Rollback)</v>
+        <v>Kiểm thử chức năng chuẩn (Happy Path)</v>
       </c>
       <c r="D19" t="str" xml:space="preserve">
         <v xml:space="preserve">1. Thiết lập phiên đăng nhập / Mock quyền truy cập tương ứng.
@@ -6553,21 +7433,21 @@
 3. Xác thực mã trạng thái HTTP và cấu trúc JSON trả về.</v>
       </c>
       <c r="E19" t="str">
-        <v>{ username: 'newuser', email: 'existing@example.com', password: 'Password123@', }</v>
+        <v>{ username: 'validuser', email: 'valid@example.com', password: 'Password123@', }</v>
       </c>
       <c r="F19" t="str">
-        <v>HTTP Status: 200. Response trả về success = true cùng dữ liệu hợp lệ.</v>
+        <v>HTTP Status: 201. Response trả về success = true cùng dữ liệu hợp lệ.</v>
       </c>
     </row>
     <row r="20" xml:space="preserve">
       <c r="A20" t="str">
-        <v>AUTH-IT-07</v>
+        <v>AUTH-IT-02</v>
       </c>
       <c r="B20" t="str">
-        <v>POST /api/auth/login khi DB mất kết nối trả về 500 lỗi máy chủ</v>
+        <v>POST /api/auth/login thành công với mã 200</v>
       </c>
       <c r="C20" t="str">
-        <v>Kiểm thử mất kết nối mạng &amp; Lỗi hệ thống (Network &amp; System Error)</v>
+        <v>Kiểm thử chức năng chuẩn (Happy Path)</v>
       </c>
       <c r="D20" t="str" xml:space="preserve">
         <v xml:space="preserve">1. Thiết lập phiên đăng nhập / Mock quyền truy cập tương ứng.
@@ -6575,15 +7455,235 @@
 3. Xác thực mã trạng thái HTTP và cấu trúc JSON trả về.</v>
       </c>
       <c r="E20" t="str">
-        <v>{ identifier: 'user@example.com', password: 'Password123@', }</v>
+        <v>{ identifier: 'valid@example.com', password: 'Password123@', }</v>
       </c>
       <c r="F20" t="str">
         <v>HTTP Status: 200. Response trả về success = true cùng dữ liệu hợp lệ.</v>
       </c>
     </row>
+    <row r="21" xml:space="preserve">
+      <c r="A21" t="str">
+        <v>AUTH-IT-02b</v>
+      </c>
+      <c r="B21" t="str">
+        <v>POST /api/auth/logout thành công khi gửi đúng token hợp lệ</v>
+      </c>
+      <c r="C21" t="str">
+        <v>Kiểm thử chức năng chuẩn (Happy Path)</v>
+      </c>
+      <c r="D21" t="str" xml:space="preserve">
+        <v xml:space="preserve">1. Thiết lập phiên đăng nhập / Mock quyền truy cập tương ứng.
+2. Gửi request HTTP POST tới endpoint /api/auth/logout.
+3. Xác thực mã trạng thái HTTP và cấu trúc JSON trả về.</v>
+      </c>
+      <c r="E21" t="str">
+        <v>{ refreshToken: 'valid_refresh_token' }</v>
+      </c>
+      <c r="F21" t="str">
+        <v>HTTP Status: 200. Response trả về success = true cùng dữ liệu hợp lệ.</v>
+      </c>
+    </row>
+    <row r="22" xml:space="preserve">
+      <c r="A22" t="str">
+        <v>AUTH-IT-03</v>
+      </c>
+      <c r="B22" t="str">
+        <v>POST /api/auth/login thiếu mật khẩu trả về 422 Validation Error</v>
+      </c>
+      <c r="C22" t="str">
+        <v>Kiểm thử trường hợp biên &amp; Ngoại lệ (Negative / Bad Case)</v>
+      </c>
+      <c r="D22" t="str" xml:space="preserve">
+        <v xml:space="preserve">1. Thiết lập phiên đăng nhập / Mock quyền truy cập tương ứng.
+2. Gửi request HTTP POST tới endpoint /api/auth/login.
+3. Xác thực mã trạng thái HTTP và cấu trúc JSON trả về.</v>
+      </c>
+      <c r="E22" t="str">
+        <v>{ identifier: 'valid@example.com', }</v>
+      </c>
+      <c r="F22" t="str">
+        <v>HTTP Status: 422. Báo lỗi validation hoặc bad request rõ ràng, không làm crash server.</v>
+      </c>
+    </row>
+    <row r="23" xml:space="preserve">
+      <c r="A23" t="str">
+        <v>AUTH-IT-04</v>
+      </c>
+      <c r="B23" t="str">
+        <v>POST /api/auth/register email không đúng định dạng trả về 422</v>
+      </c>
+      <c r="C23" t="str">
+        <v>Kiểm thử trường hợp biên &amp; Ngoại lệ (Negative / Bad Case)</v>
+      </c>
+      <c r="D23" t="str" xml:space="preserve">
+        <v xml:space="preserve">1. Thiết lập phiên đăng nhập / Mock quyền truy cập tương ứng.
+2. Gửi request HTTP POST tới endpoint /api/auth/register.
+3. Xác thực mã trạng thái HTTP và cấu trúc JSON trả về.</v>
+      </c>
+      <c r="E23" t="str">
+        <v>{ username: 'invalidmail', email: 'not-an-email', password: 'Password123@', }</v>
+      </c>
+      <c r="F23" t="str">
+        <v>HTTP Status: 422. Báo lỗi validation hoặc bad request rõ ràng, không làm crash server.</v>
+      </c>
+    </row>
+    <row r="24" xml:space="preserve">
+      <c r="A24" t="str">
+        <v>AUTH-IT-04b</v>
+      </c>
+      <c r="B24" t="str">
+        <v>POST /api/auth/logout không gửi header Authorization trả về 401</v>
+      </c>
+      <c r="C24" t="str">
+        <v>Kiểm thử phân quyền &amp; Bảo mật (Authorization &amp; Security 401/403)</v>
+      </c>
+      <c r="D24" t="str" xml:space="preserve">
+        <v xml:space="preserve">1. Thiết lập phiên đăng nhập / Mock quyền truy cập tương ứng.
+2. Gửi request HTTP POST tới endpoint /api/auth/logout.
+3. Xác thực mã trạng thái HTTP và cấu trúc JSON trả về.</v>
+      </c>
+      <c r="E24" t="str">
+        <v>{ refreshToken: 'some_refresh_token' }</v>
+      </c>
+      <c r="F24" t="str">
+        <v>HTTP Status: 401. Báo lỗi unauthorized do chưa cung cấp token xác thực.</v>
+      </c>
+    </row>
+    <row r="25" xml:space="preserve">
+      <c r="A25" t="str">
+        <v>AUTH-IT-SEC-01</v>
+      </c>
+      <c r="B25" t="str">
+        <v>Kẻ tấn công dùng Access Token đã bị thu hồi (đã logout) -&gt; Bị Authenticate middleware chặn với HTTP 401 token_revoked</v>
+      </c>
+      <c r="C25" t="str">
+        <v>Kiểm thử phân quyền &amp; Bảo mật (Authorization &amp; Security 401/403)</v>
+      </c>
+      <c r="D25" t="str" xml:space="preserve">
+        <v xml:space="preserve">1. Thiết lập phiên đăng nhập / Mock quyền truy cập tương ứng.
+2. Gửi request HTTP GET tới endpoint /api/....
+3. Xác thực mã trạng thái HTTP và cấu trúc JSON trả về.</v>
+      </c>
+      <c r="E25" t="str">
+        <v>{ refreshToken: 'any_refresh' }</v>
+      </c>
+      <c r="F25" t="str">
+        <v>HTTP Status: 401. Báo lỗi unauthorized do chưa cung cấp token xác thực.</v>
+      </c>
+    </row>
+    <row r="26" xml:space="preserve">
+      <c r="A26" t="str">
+        <v>AUTH-IT-SEC-02</v>
+      </c>
+      <c r="B26" t="str">
+        <v>Kẻ tấn công dùng Refresh Token từ session đã bị thu hồi gọi POST /api/auth/refresh -&gt; Bị chặn với HTTP 401 token_revoked</v>
+      </c>
+      <c r="C26" t="str">
+        <v>Kiểm thử phân quyền &amp; Bảo mật (Authorization &amp; Security 401/403)</v>
+      </c>
+      <c r="D26" t="str" xml:space="preserve">
+        <v xml:space="preserve">1. Thiết lập phiên đăng nhập / Mock quyền truy cập tương ứng.
+2. Gửi request HTTP POST tới endpoint /api/auth/refresh.
+3. Xác thực mã trạng thái HTTP và cấu trúc JSON trả về.</v>
+      </c>
+      <c r="E26" t="str">
+        <v>{ refreshToken: 'revoked_session_refresh_token' }</v>
+      </c>
+      <c r="F26" t="str">
+        <v>HTTP Status: 401. Báo lỗi unauthorized do chưa cung cấp token xác thực.</v>
+      </c>
+    </row>
+    <row r="27" xml:space="preserve">
+      <c r="A27" t="str">
+        <v>AUTH-IT-SEC-03</v>
+      </c>
+      <c r="B27" t="str">
+        <v>Kẻ tấn công spam Refresh Token &gt; 3 lần/phút -&gt; Hệ thống kích hoạt phòng vệ chặn 429 và hủy toàn bộ phiên</v>
+      </c>
+      <c r="C27" t="str">
+        <v>Kiểm thử phân quyền &amp; Bảo mật (Authorization &amp; Security 401/403)</v>
+      </c>
+      <c r="D27" t="str" xml:space="preserve">
+        <v xml:space="preserve">1. Thiết lập phiên đăng nhập / Mock quyền truy cập tương ứng.
+2. Gửi request HTTP GET tới endpoint /api/....
+3. Xác thực mã trạng thái HTTP và cấu trúc JSON trả về.</v>
+      </c>
+      <c r="E27" t="str">
+        <v>{ refreshToken: 'spam_refresh_token' }</v>
+      </c>
+      <c r="F27" t="str">
+        <v xml:space="preserve">HTTP Status: 429. </v>
+      </c>
+    </row>
+    <row r="28" xml:space="preserve">
+      <c r="A28" t="str">
+        <v>AUTH-IT-SEC-04</v>
+      </c>
+      <c r="B28" t="str">
+        <v>Kẻ tấn công dùng Token hợp lệ nhưng tài khoản vừa bị Admin khóa -&gt; Bị chặn với HTTP 403 account_locked ngay lập tức</v>
+      </c>
+      <c r="C28" t="str">
+        <v>Kiểm thử phân quyền &amp; Bảo mật (Authorization &amp; Security 401/403)</v>
+      </c>
+      <c r="D28" t="str" xml:space="preserve">
+        <v xml:space="preserve">1. Thiết lập phiên đăng nhập / Mock quyền truy cập tương ứng.
+2. Gửi request HTTP GET tới endpoint /api/....
+3. Xác thực mã trạng thái HTTP và cấu trúc JSON trả về.</v>
+      </c>
+      <c r="E28" t="str">
+        <v>{ refreshToken: 'any_refresh' }</v>
+      </c>
+      <c r="F28" t="str">
+        <v>HTTP Status: 403. Báo lỗi forbidden do tài khoản không có quyền truy cập thông tin quản trị.</v>
+      </c>
+    </row>
+    <row r="29" xml:space="preserve">
+      <c r="A29" t="str">
+        <v>AUTH-IT-06</v>
+      </c>
+      <c r="B29" t="str">
+        <v>POST /api/auth/register khi email đã tồn tại trả về 409 Conflict</v>
+      </c>
+      <c r="C29" t="str">
+        <v>Kiểm thử toàn vẹn dữ liệu &amp; Xung đột (Data Conflict / Rollback)</v>
+      </c>
+      <c r="D29" t="str" xml:space="preserve">
+        <v xml:space="preserve">1. Thiết lập phiên đăng nhập / Mock quyền truy cập tương ứng.
+2. Gửi request HTTP POST tới endpoint /api/auth/register.
+3. Xác thực mã trạng thái HTTP và cấu trúc JSON trả về.</v>
+      </c>
+      <c r="E29" t="str">
+        <v>{ username: 'newuser', email: 'existing@example.com', password: 'Password123@', }</v>
+      </c>
+      <c r="F29" t="str">
+        <v xml:space="preserve">HTTP Status: 409. </v>
+      </c>
+    </row>
+    <row r="30" xml:space="preserve">
+      <c r="A30" t="str">
+        <v>AUTH-IT-07</v>
+      </c>
+      <c r="B30" t="str">
+        <v>POST /api/auth/login khi DB mất kết nối trả về 500 lỗi máy chủ</v>
+      </c>
+      <c r="C30" t="str">
+        <v>Kiểm thử trường hợp biên &amp; Ngoại lệ (Negative / Bad Case)</v>
+      </c>
+      <c r="D30" t="str" xml:space="preserve">
+        <v xml:space="preserve">1. Thiết lập phiên đăng nhập / Mock quyền truy cập tương ứng.
+2. Gửi request HTTP POST tới endpoint /api/auth/login.
+3. Xác thực mã trạng thái HTTP và cấu trúc JSON trả về.</v>
+      </c>
+      <c r="E30" t="str">
+        <v>{ identifier: 'user@example.com', password: 'Password123@', }</v>
+      </c>
+      <c r="F30" t="str">
+        <v>HTTP Status: 500. Hệ thống bắt lỗi thông qua error-handler, trả về HTTP 500 an toàn.</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:F20"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:F30"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -6592,12 +7692,12 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:F14"/>
   <cols>
-    <col min="1" max="1" width="15.83203125" customWidth="1"/>
-    <col min="2" max="2" width="45.83203125" customWidth="1"/>
-    <col min="3" max="3" width="35.83203125" customWidth="1"/>
+    <col min="1" max="1" width="18.83203125" customWidth="1"/>
+    <col min="2" max="2" width="48.83203125" customWidth="1"/>
+    <col min="3" max="3" width="40.83203125" customWidth="1"/>
     <col min="4" max="4" width="45.83203125" customWidth="1"/>
     <col min="5" max="5" width="35.83203125" customWidth="1"/>
-    <col min="6" max="6" width="45.83203125" customWidth="1"/>
+    <col min="6" max="6" width="48.83203125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -6675,12 +7775,12 @@
         <v>Kiểm thử chức năng chuẩn (Happy Path)</v>
       </c>
       <c r="D4" t="str" xml:space="preserve">
-        <v xml:space="preserve">1. Khởi tạo Service với Mock Repository / Prisma Client.
-2. Kích hoạt hàm nghiệp vụ tương ứng của bubble-game.
-3. Kiểm tra giá trị trả về hoặc bắt exception.</v>
+        <v xml:space="preserve">1. Thiết lập Mock Repository / Database cho Service.
+2. Gọi method service.finishGame() với tham số kiểm thử.
+3. Đối soát kết quả hoặc mã lỗi phát sinh.</v>
       </c>
       <c r="E4" t="str">
-        <v>Dữ liệu test fixture trong bubble-game.mock.ts</v>
+        <v>Args: 1, mockFinishGameInput</v>
       </c>
       <c r="F4" t="str">
         <v>Hàm thực thi thành công, trả về đúng kiểu dữ liệu, các phương thức mock được gọi đúng tham số.</v>
@@ -6738,7 +7838,7 @@
         <v>Hai request chốt điểm finishGame gửi đồng thời</v>
       </c>
       <c r="C7" t="str">
-        <v>Kiểm thử mất kết nối mạng &amp; Lỗi hệ thống (Network &amp; System Error)</v>
+        <v>Kiểm thử đụng độ đồng thời (Concurrency / Race Condition - Update vs Delete)</v>
       </c>
       <c r="D7" t="str" xml:space="preserve">
         <v xml:space="preserve">1. Thiết lập Mock Repository / Database cho Service.
@@ -6749,7 +7849,7 @@
         <v>Args: 1, mockFinishGameInput</v>
       </c>
       <c r="F7" t="str">
-        <v>Ném ngoại lệ lỗi kết nối hoặc Rollback Transaction, không lưu dữ liệu rác.</v>
+        <v>Hệ thống phân giải đụng độ an toàn: phát hiện bản ghi đã bị xóa (P2025/404) hoặc cập nhật nguyên tử, không sinh trạng thái zombie.</v>
       </c>
     </row>
     <row r="8" xml:space="preserve">
@@ -6760,7 +7860,7 @@
         <v>Mất kết nối DB khi lưu tiến trình ném lỗi</v>
       </c>
       <c r="C8" t="str">
-        <v>Kiểm thử mất kết nối mạng &amp; Lỗi hệ thống (Network &amp; System Error)</v>
+        <v>Kiểm thử đụng độ đồng thời (Concurrency / Race Condition - Update vs Delete)</v>
       </c>
       <c r="D8" t="str" xml:space="preserve">
         <v xml:space="preserve">1. Thiết lập Mock Repository / Database cho Service.
@@ -6786,11 +7886,11 @@
       </c>
       <c r="D9" t="str" xml:space="preserve">
         <v xml:space="preserve">1. Thiết lập phiên đăng nhập / Mock quyền truy cập tương ứng.
-2. Gửi request HTTP GET tới endpoint /api/bubble-game/start.
+2. Gửi request HTTP GET tới endpoint /api/bubble-game/start?limit=4.
 3. Xác thực mã trạng thái HTTP và cấu trúc JSON trả về.</v>
       </c>
       <c r="E9" t="str">
-        <v>Path param hoặc Payload chuẩn của bubble-game</v>
+        <v>Query parameters: limit=4</v>
       </c>
       <c r="F9" t="str">
         <v>HTTP Status: 200. Response trả về success = true cùng dữ liệu hợp lệ.</v>
@@ -6812,7 +7912,7 @@
 3. Xác thực mã trạng thái HTTP và cấu trúc JSON trả về.</v>
       </c>
       <c r="E10" t="str">
-        <v>Path param hoặc Payload chuẩn của bubble-game</v>
+        <v>mockMatchPairInput</v>
       </c>
       <c r="F10" t="str">
         <v>HTTP Status: 200. Response trả về success = true cùng dữ liệu hợp lệ.</v>
@@ -6892,7 +7992,7 @@
         <v>Lỗi database khi kết thúc ván trả về 500</v>
       </c>
       <c r="C14" t="str">
-        <v>Kiểm thử mất kết nối mạng &amp; Lỗi hệ thống (Network &amp; System Error)</v>
+        <v>Kiểm thử trường hợp biên &amp; Ngoại lệ (Negative / Bad Case)</v>
       </c>
       <c r="D14" t="str" xml:space="preserve">
         <v xml:space="preserve">1. Thiết lập phiên đăng nhập / Mock quyền truy cập tương ứng.
@@ -6917,12 +8017,12 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:F18"/>
   <cols>
-    <col min="1" max="1" width="15.83203125" customWidth="1"/>
-    <col min="2" max="2" width="45.83203125" customWidth="1"/>
-    <col min="3" max="3" width="35.83203125" customWidth="1"/>
+    <col min="1" max="1" width="18.83203125" customWidth="1"/>
+    <col min="2" max="2" width="48.83203125" customWidth="1"/>
+    <col min="3" max="3" width="40.83203125" customWidth="1"/>
     <col min="4" max="4" width="45.83203125" customWidth="1"/>
     <col min="5" max="5" width="35.83203125" customWidth="1"/>
-    <col min="6" max="6" width="45.83203125" customWidth="1"/>
+    <col min="6" max="6" width="48.83203125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -7085,7 +8185,7 @@
         <v>Chỉnh sửa bài viết của người khác ném lỗi 403</v>
       </c>
       <c r="C8" t="str">
-        <v>Kiểm thử trường hợp biên &amp; Ngoại lệ (Negative / Bad Case)</v>
+        <v>Kiểm thử phân quyền &amp; Bảo mật (Authorization &amp; Security 401/403)</v>
       </c>
       <c r="D8" t="str" xml:space="preserve">
         <v xml:space="preserve">1. Thiết lập Mock Repository / Database cho Service.
@@ -7107,7 +8207,7 @@
         <v>Xóa bài viết của người khác ném lỗi 403</v>
       </c>
       <c r="C9" t="str">
-        <v>Kiểm thử trường hợp biên &amp; Ngoại lệ (Negative / Bad Case)</v>
+        <v>Kiểm thử phân quyền &amp; Bảo mật (Authorization &amp; Security 401/403)</v>
       </c>
       <c r="D9" t="str" xml:space="preserve">
         <v xml:space="preserve">1. Thiết lập Mock Repository / Database cho Service.
@@ -7129,7 +8229,7 @@
         <v>Hai request toggle like đồng thời xử lý nhất quán</v>
       </c>
       <c r="C10" t="str">
-        <v>Kiểm thử mất kết nối mạng &amp; Lỗi hệ thống (Network &amp; System Error)</v>
+        <v>Kiểm thử đụng độ đồng thời (Concurrency / Race Condition - Update vs Delete)</v>
       </c>
       <c r="D10" t="str" xml:space="preserve">
         <v xml:space="preserve">1. Thiết lập Mock Repository / Database cho Service.
@@ -7140,7 +8240,7 @@
         <v>Args: 1, 1</v>
       </c>
       <c r="F10" t="str">
-        <v>Ném ngoại lệ lỗi kết nối hoặc Rollback Transaction, không lưu dữ liệu rác.</v>
+        <v>Hệ thống phân giải đụng độ an toàn: phát hiện bản ghi đã bị xóa (P2025/404) hoặc cập nhật nguyên tử, không sinh trạng thái zombie.</v>
       </c>
     </row>
     <row r="11" xml:space="preserve">
@@ -7151,7 +8251,7 @@
         <v>Mất kết nối DB khi lấy danh sách posts ném lỗi</v>
       </c>
       <c r="C11" t="str">
-        <v>Kiểm thử mất kết nối mạng &amp; Lỗi hệ thống (Network &amp; System Error)</v>
+        <v>Kiểm thử đụng độ đồng thời (Concurrency / Race Condition - Update vs Delete)</v>
       </c>
       <c r="D11" t="str" xml:space="preserve">
         <v xml:space="preserve">1. Thiết lập Mock Repository / Database cho Service.
@@ -7177,11 +8277,11 @@
       </c>
       <c r="D12" t="str" xml:space="preserve">
         <v xml:space="preserve">1. Thiết lập phiên đăng nhập / Mock quyền truy cập tương ứng.
-2. Gửi request HTTP GET tới endpoint /api/community/posts.
+2. Gửi request HTTP GET tới endpoint /api/community/posts?page=1&amp;limit=10.
 3. Xác thực mã trạng thái HTTP và cấu trúc JSON trả về.</v>
       </c>
       <c r="E12" t="str">
-        <v>Path param hoặc Payload chuẩn của community</v>
+        <v>Query parameters: page=1&amp;limit=10</v>
       </c>
       <c r="F12" t="str">
         <v>HTTP Status: 200. Response trả về success = true cùng dữ liệu hợp lệ.</v>
@@ -7330,12 +8430,12 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:F11"/>
   <cols>
-    <col min="1" max="1" width="15.83203125" customWidth="1"/>
-    <col min="2" max="2" width="45.83203125" customWidth="1"/>
-    <col min="3" max="3" width="35.83203125" customWidth="1"/>
+    <col min="1" max="1" width="18.83203125" customWidth="1"/>
+    <col min="2" max="2" width="48.83203125" customWidth="1"/>
+    <col min="3" max="3" width="40.83203125" customWidth="1"/>
     <col min="4" max="4" width="45.83203125" customWidth="1"/>
     <col min="5" max="5" width="35.83203125" customWidth="1"/>
-    <col min="6" max="6" width="45.83203125" customWidth="1"/>
+    <col min="6" max="6" width="48.83203125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -7369,12 +8469,12 @@
         <v>Kiểm thử chức năng chuẩn (Happy Path)</v>
       </c>
       <c r="D2" t="str" xml:space="preserve">
-        <v xml:space="preserve">1. Khởi tạo Service với Mock Repository / Prisma Client.
-2. Kích hoạt hàm nghiệp vụ tương ứng của course.
-3. Kiểm tra giá trị trả về hoặc bắt exception.</v>
+        <v xml:space="preserve">1. Thiết lập Mock Repository / Database cho Service.
+2. Gọi method service.getCoursesList() với tham số kiểm thử.
+3. Đối soát kết quả hoặc mã lỗi phát sinh.</v>
       </c>
       <c r="E2" t="str">
-        <v>Dữ liệu test fixture trong course.mock.ts</v>
+        <v>Args: { page: 1, limit: 10 } as any</v>
       </c>
       <c r="F2" t="str">
         <v>Hàm thực thi thành công, trả về đúng kiểu dữ liệu, các phương thức mock được gọi đúng tham số.</v>
@@ -7391,12 +8491,12 @@
         <v>Kiểm thử chức năng chuẩn (Happy Path)</v>
       </c>
       <c r="D3" t="str" xml:space="preserve">
-        <v xml:space="preserve">1. Khởi tạo Service với Mock Repository / Prisma Client.
-2. Kích hoạt hàm nghiệp vụ tương ứng của course.
-3. Kiểm tra giá trị trả về hoặc bắt exception.</v>
+        <v xml:space="preserve">1. Thiết lập Mock Repository / Database cho Service.
+2. Gọi method service.createCourse() với tham số kiểm thử.
+3. Đối soát kết quả hoặc mã lỗi phát sinh.</v>
       </c>
       <c r="E3" t="str">
-        <v>Dữ liệu test fixture trong course.mock.ts</v>
+        <v>Args: mockCreateCourseInput as any</v>
       </c>
       <c r="F3" t="str">
         <v>Hàm thực thi thành công, trả về đúng kiểu dữ liệu, các phương thức mock được gọi đúng tham số.</v>
@@ -7454,7 +8554,7 @@
         <v>Nhiều request xóa mềm và khôi phục song song</v>
       </c>
       <c r="C6" t="str">
-        <v>Kiểm thử đụng độ đồng thời (Concurrency / Race Condition)</v>
+        <v>Kiểm thử đụng độ đồng thời (Concurrency / Race Condition - Update vs Delete)</v>
       </c>
       <c r="D6" t="str" xml:space="preserve">
         <v xml:space="preserve">1. Thiết lập Mock Repository / Database cho Service.
@@ -7465,7 +8565,7 @@
         <v>Args: 1</v>
       </c>
       <c r="F6" t="str">
-        <v>Hàm thực thi thành công, trả về đúng kiểu dữ liệu, các phương thức mock được gọi đúng tham số.</v>
+        <v>Hệ thống phân giải đụng độ an toàn: phát hiện bản ghi đã bị xóa (P2025/404) hoặc cập nhật nguyên tử, không sinh trạng thái zombie.</v>
       </c>
     </row>
     <row r="7" xml:space="preserve">
@@ -7476,7 +8576,7 @@
         <v>Mất kết nối DB khi tạo bài học ném lỗi hệ thống</v>
       </c>
       <c r="C7" t="str">
-        <v>Kiểm thử mất kết nối mạng &amp; Lỗi hệ thống (Network &amp; System Error)</v>
+        <v>Kiểm thử toàn vẹn dữ liệu &amp; Xung đột (Data Conflict / Rollback)</v>
       </c>
       <c r="D7" t="str" xml:space="preserve">
         <v xml:space="preserve">1. Thiết lập Mock Repository / Database cho Service.
@@ -7502,11 +8602,11 @@
       </c>
       <c r="D8" t="str" xml:space="preserve">
         <v xml:space="preserve">1. Thiết lập phiên đăng nhập / Mock quyền truy cập tương ứng.
-2. Gửi request HTTP GET tới endpoint /api/admin/courses.
+2. Gửi request HTTP GET tới endpoint /api/admin/courses?page=1&amp;limit=10.
 3. Xác thực mã trạng thái HTTP và cấu trúc JSON trả về.</v>
       </c>
       <c r="E8" t="str">
-        <v>Path param hoặc Payload chuẩn của course</v>
+        <v>Query parameters: page=1&amp;limit=10</v>
       </c>
       <c r="F8" t="str">
         <v>HTTP Status: 200. Response trả về success = true cùng dữ liệu hợp lệ.</v>
@@ -7589,12 +8689,12 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:F7"/>
   <cols>
-    <col min="1" max="1" width="15.83203125" customWidth="1"/>
-    <col min="2" max="2" width="45.83203125" customWidth="1"/>
-    <col min="3" max="3" width="35.83203125" customWidth="1"/>
+    <col min="1" max="1" width="18.83203125" customWidth="1"/>
+    <col min="2" max="2" width="48.83203125" customWidth="1"/>
+    <col min="3" max="3" width="40.83203125" customWidth="1"/>
     <col min="4" max="4" width="45.83203125" customWidth="1"/>
     <col min="5" max="5" width="35.83203125" customWidth="1"/>
-    <col min="6" max="6" width="45.83203125" customWidth="1"/>
+    <col min="6" max="6" width="48.83203125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -7669,7 +8769,7 @@
         <v>Nhiều Admin cùng xem Dashboard đồng thời</v>
       </c>
       <c r="C4" t="str">
-        <v>Kiểm thử đụng độ đồng thời (Concurrency / Race Condition)</v>
+        <v>Kiểm thử đụng độ đồng thời (Concurrency / Race Condition - Update vs Delete)</v>
       </c>
       <c r="D4" t="str" xml:space="preserve">
         <v xml:space="preserve">1. Thiết lập Mock Repository / Database cho Service.
@@ -7680,7 +8780,7 @@
         <v>Dữ liệu mock chuẩn của module dashboard</v>
       </c>
       <c r="F4" t="str">
-        <v>Hàm thực thi thành công, trả về đúng kiểu dữ liệu, các phương thức mock được gọi đúng tham số.</v>
+        <v>Hệ thống phân giải đụng độ an toàn: phát hiện bản ghi đã bị xóa (P2025/404) hoặc cập nhật nguyên tử, không sinh trạng thái zombie.</v>
       </c>
     </row>
     <row r="5" xml:space="preserve">
@@ -7691,7 +8791,7 @@
         <v>Mất kết nối DB khi truy vấn Dashboard ném lỗi 500</v>
       </c>
       <c r="C5" t="str">
-        <v>Kiểm thử mất kết nối mạng &amp; Lỗi hệ thống (Network &amp; System Error)</v>
+        <v>Kiểm thử toàn vẹn dữ liệu &amp; Xung đột (Data Conflict / Rollback)</v>
       </c>
       <c r="D5" t="str" xml:space="preserve">
         <v xml:space="preserve">1. Thiết lập Mock Repository / Database cho Service.

</xml_diff>